<commit_message>
Rename Section->Category (move to col B), green Today line, swimlane dividers
Template: regenerate from the original workbook with a "Category" column
inserted at B (after Task) instead of "Section" at G. Insert-at-B is a
uniform right-shift of columns >= B, so all CF ranges, formulas, merges,
the StartAbs name, and the Milestone checkbox column (E->F) remap cleanly;
protection and modern features preserved. Final layout:
Task | Category | Status | Start | End | Milestone | Notes | sprints…

App:
- Parser detects a "Category" (or "Section") header; task table column
  renamed to Category.
- Now line is now solid green and labelled "Today" (preview + PPTX).
- Thin grey divider lines drawn between section swimlanes (preview + PPTX).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WPLuxHLXTyjEHoQp8LTD3B
</commit_message>
<xml_diff>
--- a/assets/delivery-plan-template.xlsx
+++ b/assets/delivery-plan-template.xlsx
@@ -1004,11 +1004,11 @@
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="4" width="12.28515625" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" customWidth="1"/>
-    <col min="6" max="6" width="36" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="5" width="12.28515625" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" customWidth="1"/>
+    <col min="7" max="7" width="36" customWidth="1"/>
     <col min="8" max="35" width="6.42578125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1016,11 +1016,11 @@
       <c r="A1" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="27"/>
       <c r="C1" s="27"/>
       <c r="D1" s="27"/>
       <c r="E1" s="27"/>
       <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
       <c r="H1" s="10" t="s">
         <v>0</v>
       </c>
@@ -1044,35 +1044,35 @@
     </row>
     <row r="2" spans="1:35" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="23"/>
-      <c r="B2" s="23"/>
       <c r="C2" s="23"/>
       <c r="D2" s="23"/>
       <c r="E2" s="23"/>
       <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
     </row>
     <row r="3" spans="1:35" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="D3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="E3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="F3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="G3" s="7" t="s">
         <v>6</v>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
       </c>
       <c r="H3" s="8" t="str">
         <f>("Q"&amp;(MOD(INT((StartAbs+0-1)/7),4)+1)&amp;"."&amp;(MOD(StartAbs+0-1,7)+1))</f>
@@ -1189,137 +1189,137 @@
     </row>
     <row r="4" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="16"/>
-      <c r="B4" s="17"/>
+      <c r="B4" s="16"/>
       <c r="C4" s="17"/>
       <c r="D4" s="17"/>
-      <c r="E4" s="18" t="b">
+      <c r="E4" s="17"/>
+      <c r="F4" s="18" t="b">
         <v>0</v>
       </c>
-      <c r="F4" s="16"/>
       <c r="G4" s="16"/>
       <c r="H4" s="5" t="str">
-        <f t="shared" ref="H4:H35" si="0">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=1,MATCH($D4,$H$3:$AI$3,0)&gt;=1),1,""),"")</f>
+        <f t="shared" ref="H4:H35" si="0">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=1,MATCH($E4,$H$3:$AI$3,0)&gt;=1),1,""),"")</f>
         <v/>
       </c>
       <c r="I4" s="6" t="str">
-        <f t="shared" ref="I4:I35" si="1">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=2,MATCH($D4,$H$3:$AI$3,0)&gt;=2),1,""),"")</f>
+        <f t="shared" ref="I4:I35" si="1">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=2,MATCH($E4,$H$3:$AI$3,0)&gt;=2),1,""),"")</f>
         <v/>
       </c>
       <c r="J4" s="6" t="str">
-        <f t="shared" ref="J4:J35" si="2">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=3,MATCH($D4,$H$3:$AI$3,0)&gt;=3),1,""),"")</f>
+        <f t="shared" ref="J4:J35" si="2">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=3,MATCH($E4,$H$3:$AI$3,0)&gt;=3),1,""),"")</f>
         <v/>
       </c>
       <c r="K4" s="6" t="str">
-        <f t="shared" ref="K4:K35" si="3">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=4,MATCH($D4,$H$3:$AI$3,0)&gt;=4),1,""),"")</f>
+        <f t="shared" ref="K4:K35" si="3">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=4,MATCH($E4,$H$3:$AI$3,0)&gt;=4),1,""),"")</f>
         <v/>
       </c>
       <c r="L4" s="6" t="str">
-        <f t="shared" ref="L4:L35" si="4">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=5,MATCH($D4,$H$3:$AI$3,0)&gt;=5),1,""),"")</f>
+        <f t="shared" ref="L4:L35" si="4">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=5,MATCH($E4,$H$3:$AI$3,0)&gt;=5),1,""),"")</f>
         <v/>
       </c>
       <c r="M4" s="6" t="str">
-        <f t="shared" ref="M4:M35" si="5">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=6,MATCH($D4,$H$3:$AI$3,0)&gt;=6),1,""),"")</f>
+        <f t="shared" ref="M4:M35" si="5">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=6,MATCH($E4,$H$3:$AI$3,0)&gt;=6),1,""),"")</f>
         <v/>
       </c>
       <c r="N4" s="6" t="str">
-        <f t="shared" ref="N4:N35" si="6">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=7,MATCH($D4,$H$3:$AI$3,0)&gt;=7),1,""),"")</f>
+        <f t="shared" ref="N4:N35" si="6">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=7,MATCH($E4,$H$3:$AI$3,0)&gt;=7),1,""),"")</f>
         <v/>
       </c>
       <c r="O4" s="6" t="str">
-        <f t="shared" ref="O4:O35" si="7">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=8,MATCH($D4,$H$3:$AI$3,0)&gt;=8),1,""),"")</f>
+        <f t="shared" ref="O4:O35" si="7">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=8,MATCH($E4,$H$3:$AI$3,0)&gt;=8),1,""),"")</f>
         <v/>
       </c>
       <c r="P4" s="6" t="str">
-        <f t="shared" ref="P4:P35" si="8">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=9,MATCH($D4,$H$3:$AI$3,0)&gt;=9),1,""),"")</f>
+        <f t="shared" ref="P4:P35" si="8">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=9,MATCH($E4,$H$3:$AI$3,0)&gt;=9),1,""),"")</f>
         <v/>
       </c>
       <c r="Q4" s="6" t="str">
-        <f t="shared" ref="Q4:Q35" si="9">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=10,MATCH($D4,$H$3:$AI$3,0)&gt;=10),1,""),"")</f>
+        <f t="shared" ref="Q4:Q35" si="9">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=10,MATCH($E4,$H$3:$AI$3,0)&gt;=10),1,""),"")</f>
         <v/>
       </c>
       <c r="R4" s="6" t="str">
-        <f t="shared" ref="R4:R35" si="10">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=11,MATCH($D4,$H$3:$AI$3,0)&gt;=11),1,""),"")</f>
+        <f t="shared" ref="R4:R35" si="10">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=11,MATCH($E4,$H$3:$AI$3,0)&gt;=11),1,""),"")</f>
         <v/>
       </c>
       <c r="S4" s="6" t="str">
-        <f t="shared" ref="S4:S35" si="11">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=12,MATCH($D4,$H$3:$AI$3,0)&gt;=12),1,""),"")</f>
+        <f t="shared" ref="S4:S35" si="11">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=12,MATCH($E4,$H$3:$AI$3,0)&gt;=12),1,""),"")</f>
         <v/>
       </c>
       <c r="T4" s="6" t="str">
-        <f t="shared" ref="T4:T35" si="12">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=13,MATCH($D4,$H$3:$AI$3,0)&gt;=13),1,""),"")</f>
+        <f t="shared" ref="T4:T35" si="12">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=13,MATCH($E4,$H$3:$AI$3,0)&gt;=13),1,""),"")</f>
         <v/>
       </c>
       <c r="U4" s="6" t="str">
-        <f t="shared" ref="U4:U35" si="13">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=14,MATCH($D4,$H$3:$AI$3,0)&gt;=14),1,""),"")</f>
+        <f t="shared" ref="U4:U35" si="13">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=14,MATCH($E4,$H$3:$AI$3,0)&gt;=14),1,""),"")</f>
         <v/>
       </c>
       <c r="V4" s="6" t="str">
-        <f t="shared" ref="V4:V35" si="14">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=15,MATCH($D4,$H$3:$AI$3,0)&gt;=15),1,""),"")</f>
+        <f t="shared" ref="V4:V35" si="14">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=15,MATCH($E4,$H$3:$AI$3,0)&gt;=15),1,""),"")</f>
         <v/>
       </c>
       <c r="W4" s="6" t="str">
-        <f t="shared" ref="W4:W35" si="15">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=16,MATCH($D4,$H$3:$AI$3,0)&gt;=16),1,""),"")</f>
+        <f t="shared" ref="W4:W35" si="15">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=16,MATCH($E4,$H$3:$AI$3,0)&gt;=16),1,""),"")</f>
         <v/>
       </c>
       <c r="X4" s="6" t="str">
-        <f t="shared" ref="X4:X35" si="16">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=17,MATCH($D4,$H$3:$AI$3,0)&gt;=17),1,""),"")</f>
+        <f t="shared" ref="X4:X35" si="16">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=17,MATCH($E4,$H$3:$AI$3,0)&gt;=17),1,""),"")</f>
         <v/>
       </c>
       <c r="Y4" s="6" t="str">
-        <f t="shared" ref="Y4:Y35" si="17">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=18,MATCH($D4,$H$3:$AI$3,0)&gt;=18),1,""),"")</f>
+        <f t="shared" ref="Y4:Y35" si="17">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=18,MATCH($E4,$H$3:$AI$3,0)&gt;=18),1,""),"")</f>
         <v/>
       </c>
       <c r="Z4" s="6" t="str">
-        <f t="shared" ref="Z4:Z35" si="18">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=19,MATCH($D4,$H$3:$AI$3,0)&gt;=19),1,""),"")</f>
+        <f t="shared" ref="Z4:Z35" si="18">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=19,MATCH($E4,$H$3:$AI$3,0)&gt;=19),1,""),"")</f>
         <v/>
       </c>
       <c r="AA4" s="6" t="str">
-        <f t="shared" ref="AA4:AA35" si="19">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=20,MATCH($D4,$H$3:$AI$3,0)&gt;=20),1,""),"")</f>
+        <f t="shared" ref="AA4:AA35" si="19">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=20,MATCH($E4,$H$3:$AI$3,0)&gt;=20),1,""),"")</f>
         <v/>
       </c>
       <c r="AB4" s="6" t="str">
-        <f t="shared" ref="AB4:AB35" si="20">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=21,MATCH($D4,$H$3:$AI$3,0)&gt;=21),1,""),"")</f>
+        <f t="shared" ref="AB4:AB35" si="20">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=21,MATCH($E4,$H$3:$AI$3,0)&gt;=21),1,""),"")</f>
         <v/>
       </c>
       <c r="AC4" s="6" t="str">
-        <f t="shared" ref="AC4:AC35" si="21">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=22,MATCH($D4,$H$3:$AI$3,0)&gt;=22),1,""),"")</f>
+        <f t="shared" ref="AC4:AC35" si="21">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=22,MATCH($E4,$H$3:$AI$3,0)&gt;=22),1,""),"")</f>
         <v/>
       </c>
       <c r="AD4" s="6" t="str">
-        <f t="shared" ref="AD4:AD35" si="22">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=23,MATCH($D4,$H$3:$AI$3,0)&gt;=23),1,""),"")</f>
+        <f t="shared" ref="AD4:AD35" si="22">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=23,MATCH($E4,$H$3:$AI$3,0)&gt;=23),1,""),"")</f>
         <v/>
       </c>
       <c r="AE4" s="6" t="str">
-        <f t="shared" ref="AE4:AE35" si="23">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=24,MATCH($D4,$H$3:$AI$3,0)&gt;=24),1,""),"")</f>
+        <f t="shared" ref="AE4:AE35" si="23">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=24,MATCH($E4,$H$3:$AI$3,0)&gt;=24),1,""),"")</f>
         <v/>
       </c>
       <c r="AF4" s="6" t="str">
-        <f t="shared" ref="AF4:AF35" si="24">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=25,MATCH($D4,$H$3:$AI$3,0)&gt;=25),1,""),"")</f>
+        <f t="shared" ref="AF4:AF35" si="24">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=25,MATCH($E4,$H$3:$AI$3,0)&gt;=25),1,""),"")</f>
         <v/>
       </c>
       <c r="AG4" s="6" t="str">
-        <f t="shared" ref="AG4:AG35" si="25">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=26,MATCH($D4,$H$3:$AI$3,0)&gt;=26),1,""),"")</f>
+        <f t="shared" ref="AG4:AG35" si="25">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=26,MATCH($E4,$H$3:$AI$3,0)&gt;=26),1,""),"")</f>
         <v/>
       </c>
       <c r="AH4" s="6" t="str">
-        <f t="shared" ref="AH4:AH35" si="26">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=27,MATCH($D4,$H$3:$AI$3,0)&gt;=27),1,""),"")</f>
+        <f t="shared" ref="AH4:AH35" si="26">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=27,MATCH($E4,$H$3:$AI$3,0)&gt;=27),1,""),"")</f>
         <v/>
       </c>
       <c r="AI4" s="13" t="str">
-        <f t="shared" ref="AI4:AI35" si="27">IFERROR(IF(AND(MATCH($C4,$H$3:$AI$3,0)&lt;=28,MATCH($D4,$H$3:$AI$3,0)&gt;=28),1,""),"")</f>
+        <f t="shared" ref="AI4:AI35" si="27">IFERROR(IF(AND(MATCH($D4,$H$3:$AI$3,0)&lt;=28,MATCH($E4,$H$3:$AI$3,0)&gt;=28),1,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="5" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="19"/>
-      <c r="B5" s="20"/>
+      <c r="B5" s="16"/>
       <c r="C5" s="20"/>
       <c r="D5" s="20"/>
-      <c r="E5" s="21" t="b">
+      <c r="E5" s="20"/>
+      <c r="F5" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F5" s="19"/>
-      <c r="G5" s="16"/>
+      <c r="G5" s="19"/>
       <c r="H5" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1435,14 +1435,14 @@
     </row>
     <row r="6" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19"/>
-      <c r="B6" s="20"/>
+      <c r="B6" s="16"/>
       <c r="C6" s="20"/>
       <c r="D6" s="20"/>
-      <c r="E6" s="21" t="b">
+      <c r="E6" s="20"/>
+      <c r="F6" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F6" s="19"/>
-      <c r="G6" s="16"/>
+      <c r="G6" s="19"/>
       <c r="H6" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1558,14 +1558,14 @@
     </row>
     <row r="7" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="19"/>
-      <c r="B7" s="20"/>
+      <c r="B7" s="16"/>
       <c r="C7" s="20"/>
       <c r="D7" s="20"/>
-      <c r="E7" s="21" t="b">
+      <c r="E7" s="20"/>
+      <c r="F7" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F7" s="19"/>
-      <c r="G7" s="16"/>
+      <c r="G7" s="19"/>
       <c r="H7" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1681,14 +1681,14 @@
     </row>
     <row r="8" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19"/>
-      <c r="B8" s="20"/>
+      <c r="B8" s="16"/>
       <c r="C8" s="20"/>
       <c r="D8" s="20"/>
-      <c r="E8" s="21" t="b">
+      <c r="E8" s="20"/>
+      <c r="F8" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F8" s="19"/>
-      <c r="G8" s="16"/>
+      <c r="G8" s="19"/>
       <c r="H8" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1804,14 +1804,14 @@
     </row>
     <row r="9" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="19"/>
-      <c r="B9" s="20"/>
+      <c r="B9" s="16"/>
       <c r="C9" s="20"/>
       <c r="D9" s="20"/>
-      <c r="E9" s="21" t="b">
+      <c r="E9" s="20"/>
+      <c r="F9" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F9" s="19"/>
-      <c r="G9" s="16"/>
+      <c r="G9" s="19"/>
       <c r="H9" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1927,14 +1927,14 @@
     </row>
     <row r="10" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19"/>
-      <c r="B10" s="20"/>
+      <c r="B10" s="16"/>
       <c r="C10" s="20"/>
       <c r="D10" s="20"/>
-      <c r="E10" s="21" t="b">
+      <c r="E10" s="20"/>
+      <c r="F10" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F10" s="19"/>
-      <c r="G10" s="16"/>
+      <c r="G10" s="19"/>
       <c r="H10" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2050,14 +2050,14 @@
     </row>
     <row r="11" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19"/>
-      <c r="B11" s="20"/>
+      <c r="B11" s="16"/>
       <c r="C11" s="20"/>
       <c r="D11" s="20"/>
-      <c r="E11" s="21" t="b">
+      <c r="E11" s="20"/>
+      <c r="F11" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F11" s="19"/>
-      <c r="G11" s="16"/>
+      <c r="G11" s="19"/>
       <c r="H11" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2173,14 +2173,14 @@
     </row>
     <row r="12" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="19"/>
-      <c r="B12" s="20"/>
+      <c r="B12" s="16"/>
       <c r="C12" s="20"/>
       <c r="D12" s="20"/>
-      <c r="E12" s="21" t="b">
+      <c r="E12" s="20"/>
+      <c r="F12" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F12" s="19"/>
-      <c r="G12" s="16"/>
+      <c r="G12" s="19"/>
       <c r="H12" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2296,14 +2296,14 @@
     </row>
     <row r="13" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19"/>
-      <c r="B13" s="20"/>
+      <c r="B13" s="16"/>
       <c r="C13" s="20"/>
       <c r="D13" s="20"/>
-      <c r="E13" s="21" t="b">
+      <c r="E13" s="20"/>
+      <c r="F13" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F13" s="19"/>
-      <c r="G13" s="16"/>
+      <c r="G13" s="19"/>
       <c r="H13" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2419,14 +2419,14 @@
     </row>
     <row r="14" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="19"/>
-      <c r="B14" s="20"/>
+      <c r="B14" s="16"/>
       <c r="C14" s="20"/>
       <c r="D14" s="20"/>
-      <c r="E14" s="21" t="b">
+      <c r="E14" s="20"/>
+      <c r="F14" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F14" s="19"/>
-      <c r="G14" s="16"/>
+      <c r="G14" s="19"/>
       <c r="H14" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2542,14 +2542,14 @@
     </row>
     <row r="15" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="19"/>
-      <c r="B15" s="20"/>
+      <c r="B15" s="16"/>
       <c r="C15" s="20"/>
       <c r="D15" s="20"/>
-      <c r="E15" s="21" t="b">
+      <c r="E15" s="20"/>
+      <c r="F15" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F15" s="19"/>
-      <c r="G15" s="16"/>
+      <c r="G15" s="19"/>
       <c r="H15" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2665,14 +2665,14 @@
     </row>
     <row r="16" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19"/>
-      <c r="B16" s="20"/>
+      <c r="B16" s="16"/>
       <c r="C16" s="20"/>
       <c r="D16" s="20"/>
-      <c r="E16" s="21" t="b">
+      <c r="E16" s="20"/>
+      <c r="F16" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F16" s="19"/>
-      <c r="G16" s="16"/>
+      <c r="G16" s="19"/>
       <c r="H16" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2788,14 +2788,14 @@
     </row>
     <row r="17" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="19"/>
-      <c r="B17" s="20"/>
+      <c r="B17" s="16"/>
       <c r="C17" s="20"/>
       <c r="D17" s="20"/>
-      <c r="E17" s="21" t="b">
+      <c r="E17" s="20"/>
+      <c r="F17" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F17" s="19"/>
-      <c r="G17" s="16"/>
+      <c r="G17" s="19"/>
       <c r="H17" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2911,14 +2911,14 @@
     </row>
     <row r="18" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="19"/>
-      <c r="B18" s="20"/>
+      <c r="B18" s="16"/>
       <c r="C18" s="20"/>
       <c r="D18" s="20"/>
-      <c r="E18" s="21" t="b">
+      <c r="E18" s="20"/>
+      <c r="F18" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F18" s="19"/>
-      <c r="G18" s="16"/>
+      <c r="G18" s="19"/>
       <c r="H18" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3034,14 +3034,14 @@
     </row>
     <row r="19" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="19"/>
-      <c r="B19" s="20"/>
+      <c r="B19" s="16"/>
       <c r="C19" s="20"/>
       <c r="D19" s="20"/>
-      <c r="E19" s="21" t="b">
+      <c r="E19" s="20"/>
+      <c r="F19" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F19" s="19"/>
-      <c r="G19" s="16"/>
+      <c r="G19" s="19"/>
       <c r="H19" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3157,14 +3157,14 @@
     </row>
     <row r="20" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="19"/>
-      <c r="B20" s="20"/>
+      <c r="B20" s="16"/>
       <c r="C20" s="20"/>
       <c r="D20" s="20"/>
-      <c r="E20" s="21" t="b">
+      <c r="E20" s="20"/>
+      <c r="F20" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F20" s="19"/>
-      <c r="G20" s="16"/>
+      <c r="G20" s="19"/>
       <c r="H20" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3280,14 +3280,14 @@
     </row>
     <row r="21" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="19"/>
-      <c r="B21" s="20"/>
+      <c r="B21" s="16"/>
       <c r="C21" s="20"/>
       <c r="D21" s="20"/>
-      <c r="E21" s="21" t="b">
+      <c r="E21" s="20"/>
+      <c r="F21" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F21" s="19"/>
-      <c r="G21" s="16"/>
+      <c r="G21" s="19"/>
       <c r="H21" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3403,14 +3403,14 @@
     </row>
     <row r="22" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="19"/>
-      <c r="B22" s="20"/>
+      <c r="B22" s="16"/>
       <c r="C22" s="20"/>
       <c r="D22" s="20"/>
-      <c r="E22" s="21" t="b">
+      <c r="E22" s="20"/>
+      <c r="F22" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F22" s="19"/>
-      <c r="G22" s="16"/>
+      <c r="G22" s="19"/>
       <c r="H22" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3526,14 +3526,14 @@
     </row>
     <row r="23" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="19"/>
-      <c r="B23" s="20"/>
+      <c r="B23" s="16"/>
       <c r="C23" s="20"/>
       <c r="D23" s="20"/>
-      <c r="E23" s="21" t="b">
+      <c r="E23" s="20"/>
+      <c r="F23" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F23" s="19"/>
-      <c r="G23" s="16"/>
+      <c r="G23" s="19"/>
       <c r="H23" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3649,14 +3649,14 @@
     </row>
     <row r="24" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="19"/>
-      <c r="B24" s="20"/>
+      <c r="B24" s="16"/>
       <c r="C24" s="20"/>
       <c r="D24" s="20"/>
-      <c r="E24" s="21" t="b">
+      <c r="E24" s="20"/>
+      <c r="F24" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F24" s="19"/>
-      <c r="G24" s="16"/>
+      <c r="G24" s="19"/>
       <c r="H24" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3772,14 +3772,14 @@
     </row>
     <row r="25" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="19"/>
-      <c r="B25" s="20"/>
+      <c r="B25" s="16"/>
       <c r="C25" s="20"/>
       <c r="D25" s="20"/>
-      <c r="E25" s="21" t="b">
+      <c r="E25" s="20"/>
+      <c r="F25" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F25" s="19"/>
-      <c r="G25" s="16"/>
+      <c r="G25" s="19"/>
       <c r="H25" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3895,14 +3895,14 @@
     </row>
     <row r="26" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="19"/>
-      <c r="B26" s="20"/>
+      <c r="B26" s="16"/>
       <c r="C26" s="20"/>
       <c r="D26" s="20"/>
-      <c r="E26" s="21" t="b">
+      <c r="E26" s="20"/>
+      <c r="F26" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F26" s="19"/>
-      <c r="G26" s="16"/>
+      <c r="G26" s="19"/>
       <c r="H26" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4018,14 +4018,14 @@
     </row>
     <row r="27" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="19"/>
-      <c r="B27" s="20"/>
+      <c r="B27" s="16"/>
       <c r="C27" s="20"/>
       <c r="D27" s="20"/>
-      <c r="E27" s="21" t="b">
+      <c r="E27" s="20"/>
+      <c r="F27" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F27" s="19"/>
-      <c r="G27" s="16"/>
+      <c r="G27" s="19"/>
       <c r="H27" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4141,14 +4141,14 @@
     </row>
     <row r="28" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="19"/>
-      <c r="B28" s="20"/>
+      <c r="B28" s="16"/>
       <c r="C28" s="20"/>
       <c r="D28" s="20"/>
-      <c r="E28" s="21" t="b">
+      <c r="E28" s="20"/>
+      <c r="F28" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F28" s="19"/>
-      <c r="G28" s="16"/>
+      <c r="G28" s="19"/>
       <c r="H28" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4264,14 +4264,14 @@
     </row>
     <row r="29" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="19"/>
-      <c r="B29" s="20"/>
+      <c r="B29" s="16"/>
       <c r="C29" s="20"/>
       <c r="D29" s="20"/>
-      <c r="E29" s="21" t="b">
+      <c r="E29" s="20"/>
+      <c r="F29" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F29" s="19"/>
-      <c r="G29" s="16"/>
+      <c r="G29" s="19"/>
       <c r="H29" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4387,14 +4387,14 @@
     </row>
     <row r="30" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="19"/>
-      <c r="B30" s="20"/>
+      <c r="B30" s="16"/>
       <c r="C30" s="20"/>
       <c r="D30" s="20"/>
-      <c r="E30" s="21" t="b">
+      <c r="E30" s="20"/>
+      <c r="F30" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F30" s="19"/>
-      <c r="G30" s="16"/>
+      <c r="G30" s="19"/>
       <c r="H30" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4510,14 +4510,14 @@
     </row>
     <row r="31" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="19"/>
-      <c r="B31" s="20"/>
+      <c r="B31" s="16"/>
       <c r="C31" s="20"/>
       <c r="D31" s="20"/>
-      <c r="E31" s="21" t="b">
+      <c r="E31" s="20"/>
+      <c r="F31" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F31" s="19"/>
-      <c r="G31" s="16"/>
+      <c r="G31" s="19"/>
       <c r="H31" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4633,14 +4633,14 @@
     </row>
     <row r="32" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="19"/>
-      <c r="B32" s="20"/>
+      <c r="B32" s="16"/>
       <c r="C32" s="20"/>
       <c r="D32" s="20"/>
-      <c r="E32" s="21" t="b">
+      <c r="E32" s="20"/>
+      <c r="F32" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F32" s="19"/>
-      <c r="G32" s="16"/>
+      <c r="G32" s="19"/>
       <c r="H32" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4756,14 +4756,14 @@
     </row>
     <row r="33" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="19"/>
-      <c r="B33" s="20"/>
+      <c r="B33" s="16"/>
       <c r="C33" s="20"/>
       <c r="D33" s="20"/>
-      <c r="E33" s="21" t="b">
+      <c r="E33" s="20"/>
+      <c r="F33" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F33" s="19"/>
-      <c r="G33" s="16"/>
+      <c r="G33" s="19"/>
       <c r="H33" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -4879,14 +4879,14 @@
     </row>
     <row r="34" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="19"/>
-      <c r="B34" s="20"/>
+      <c r="B34" s="16"/>
       <c r="C34" s="20"/>
       <c r="D34" s="20"/>
-      <c r="E34" s="21" t="b">
+      <c r="E34" s="20"/>
+      <c r="F34" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F34" s="19"/>
-      <c r="G34" s="16"/>
+      <c r="G34" s="19"/>
       <c r="H34" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -5002,14 +5002,14 @@
     </row>
     <row r="35" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="19"/>
-      <c r="B35" s="20"/>
+      <c r="B35" s="16"/>
       <c r="C35" s="20"/>
       <c r="D35" s="20"/>
-      <c r="E35" s="21" t="b">
+      <c r="E35" s="20"/>
+      <c r="F35" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F35" s="19"/>
-      <c r="G35" s="16"/>
+      <c r="G35" s="19"/>
       <c r="H35" s="1" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -5125,137 +5125,137 @@
     </row>
     <row r="36" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="19"/>
-      <c r="B36" s="20"/>
+      <c r="B36" s="16"/>
       <c r="C36" s="20"/>
       <c r="D36" s="20"/>
-      <c r="E36" s="21" t="b">
+      <c r="E36" s="20"/>
+      <c r="F36" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F36" s="19"/>
-      <c r="G36" s="16"/>
+      <c r="G36" s="19"/>
       <c r="H36" s="1" t="str">
-        <f t="shared" ref="H36:H67" si="28">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=1,MATCH($D36,$H$3:$AI$3,0)&gt;=1),1,""),"")</f>
+        <f t="shared" ref="H36:H67" si="28">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=1,MATCH($E36,$H$3:$AI$3,0)&gt;=1),1,""),"")</f>
         <v/>
       </c>
       <c r="I36" s="2" t="str">
-        <f t="shared" ref="I36:I67" si="29">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=2,MATCH($D36,$H$3:$AI$3,0)&gt;=2),1,""),"")</f>
+        <f t="shared" ref="I36:I67" si="29">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=2,MATCH($E36,$H$3:$AI$3,0)&gt;=2),1,""),"")</f>
         <v/>
       </c>
       <c r="J36" s="2" t="str">
-        <f t="shared" ref="J36:J67" si="30">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=3,MATCH($D36,$H$3:$AI$3,0)&gt;=3),1,""),"")</f>
+        <f t="shared" ref="J36:J67" si="30">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=3,MATCH($E36,$H$3:$AI$3,0)&gt;=3),1,""),"")</f>
         <v/>
       </c>
       <c r="K36" s="2" t="str">
-        <f t="shared" ref="K36:K67" si="31">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=4,MATCH($D36,$H$3:$AI$3,0)&gt;=4),1,""),"")</f>
+        <f t="shared" ref="K36:K67" si="31">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=4,MATCH($E36,$H$3:$AI$3,0)&gt;=4),1,""),"")</f>
         <v/>
       </c>
       <c r="L36" s="2" t="str">
-        <f t="shared" ref="L36:L67" si="32">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=5,MATCH($D36,$H$3:$AI$3,0)&gt;=5),1,""),"")</f>
+        <f t="shared" ref="L36:L67" si="32">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=5,MATCH($E36,$H$3:$AI$3,0)&gt;=5),1,""),"")</f>
         <v/>
       </c>
       <c r="M36" s="2" t="str">
-        <f t="shared" ref="M36:M67" si="33">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=6,MATCH($D36,$H$3:$AI$3,0)&gt;=6),1,""),"")</f>
+        <f t="shared" ref="M36:M67" si="33">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=6,MATCH($E36,$H$3:$AI$3,0)&gt;=6),1,""),"")</f>
         <v/>
       </c>
       <c r="N36" s="2" t="str">
-        <f t="shared" ref="N36:N67" si="34">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=7,MATCH($D36,$H$3:$AI$3,0)&gt;=7),1,""),"")</f>
+        <f t="shared" ref="N36:N67" si="34">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=7,MATCH($E36,$H$3:$AI$3,0)&gt;=7),1,""),"")</f>
         <v/>
       </c>
       <c r="O36" s="2" t="str">
-        <f t="shared" ref="O36:O67" si="35">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=8,MATCH($D36,$H$3:$AI$3,0)&gt;=8),1,""),"")</f>
+        <f t="shared" ref="O36:O67" si="35">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=8,MATCH($E36,$H$3:$AI$3,0)&gt;=8),1,""),"")</f>
         <v/>
       </c>
       <c r="P36" s="2" t="str">
-        <f t="shared" ref="P36:P67" si="36">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=9,MATCH($D36,$H$3:$AI$3,0)&gt;=9),1,""),"")</f>
+        <f t="shared" ref="P36:P67" si="36">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=9,MATCH($E36,$H$3:$AI$3,0)&gt;=9),1,""),"")</f>
         <v/>
       </c>
       <c r="Q36" s="2" t="str">
-        <f t="shared" ref="Q36:Q67" si="37">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=10,MATCH($D36,$H$3:$AI$3,0)&gt;=10),1,""),"")</f>
+        <f t="shared" ref="Q36:Q67" si="37">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=10,MATCH($E36,$H$3:$AI$3,0)&gt;=10),1,""),"")</f>
         <v/>
       </c>
       <c r="R36" s="2" t="str">
-        <f t="shared" ref="R36:R67" si="38">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=11,MATCH($D36,$H$3:$AI$3,0)&gt;=11),1,""),"")</f>
+        <f t="shared" ref="R36:R67" si="38">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=11,MATCH($E36,$H$3:$AI$3,0)&gt;=11),1,""),"")</f>
         <v/>
       </c>
       <c r="S36" s="2" t="str">
-        <f t="shared" ref="S36:S67" si="39">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=12,MATCH($D36,$H$3:$AI$3,0)&gt;=12),1,""),"")</f>
+        <f t="shared" ref="S36:S67" si="39">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=12,MATCH($E36,$H$3:$AI$3,0)&gt;=12),1,""),"")</f>
         <v/>
       </c>
       <c r="T36" s="2" t="str">
-        <f t="shared" ref="T36:T67" si="40">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=13,MATCH($D36,$H$3:$AI$3,0)&gt;=13),1,""),"")</f>
+        <f t="shared" ref="T36:T67" si="40">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=13,MATCH($E36,$H$3:$AI$3,0)&gt;=13),1,""),"")</f>
         <v/>
       </c>
       <c r="U36" s="2" t="str">
-        <f t="shared" ref="U36:U67" si="41">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=14,MATCH($D36,$H$3:$AI$3,0)&gt;=14),1,""),"")</f>
+        <f t="shared" ref="U36:U67" si="41">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=14,MATCH($E36,$H$3:$AI$3,0)&gt;=14),1,""),"")</f>
         <v/>
       </c>
       <c r="V36" s="2" t="str">
-        <f t="shared" ref="V36:V67" si="42">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=15,MATCH($D36,$H$3:$AI$3,0)&gt;=15),1,""),"")</f>
+        <f t="shared" ref="V36:V67" si="42">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=15,MATCH($E36,$H$3:$AI$3,0)&gt;=15),1,""),"")</f>
         <v/>
       </c>
       <c r="W36" s="2" t="str">
-        <f t="shared" ref="W36:W67" si="43">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=16,MATCH($D36,$H$3:$AI$3,0)&gt;=16),1,""),"")</f>
+        <f t="shared" ref="W36:W67" si="43">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=16,MATCH($E36,$H$3:$AI$3,0)&gt;=16),1,""),"")</f>
         <v/>
       </c>
       <c r="X36" s="2" t="str">
-        <f t="shared" ref="X36:X67" si="44">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=17,MATCH($D36,$H$3:$AI$3,0)&gt;=17),1,""),"")</f>
+        <f t="shared" ref="X36:X67" si="44">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=17,MATCH($E36,$H$3:$AI$3,0)&gt;=17),1,""),"")</f>
         <v/>
       </c>
       <c r="Y36" s="2" t="str">
-        <f t="shared" ref="Y36:Y67" si="45">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=18,MATCH($D36,$H$3:$AI$3,0)&gt;=18),1,""),"")</f>
+        <f t="shared" ref="Y36:Y67" si="45">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=18,MATCH($E36,$H$3:$AI$3,0)&gt;=18),1,""),"")</f>
         <v/>
       </c>
       <c r="Z36" s="2" t="str">
-        <f t="shared" ref="Z36:Z67" si="46">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=19,MATCH($D36,$H$3:$AI$3,0)&gt;=19),1,""),"")</f>
+        <f t="shared" ref="Z36:Z67" si="46">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=19,MATCH($E36,$H$3:$AI$3,0)&gt;=19),1,""),"")</f>
         <v/>
       </c>
       <c r="AA36" s="2" t="str">
-        <f t="shared" ref="AA36:AA67" si="47">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=20,MATCH($D36,$H$3:$AI$3,0)&gt;=20),1,""),"")</f>
+        <f t="shared" ref="AA36:AA67" si="47">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=20,MATCH($E36,$H$3:$AI$3,0)&gt;=20),1,""),"")</f>
         <v/>
       </c>
       <c r="AB36" s="2" t="str">
-        <f t="shared" ref="AB36:AB67" si="48">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=21,MATCH($D36,$H$3:$AI$3,0)&gt;=21),1,""),"")</f>
+        <f t="shared" ref="AB36:AB67" si="48">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=21,MATCH($E36,$H$3:$AI$3,0)&gt;=21),1,""),"")</f>
         <v/>
       </c>
       <c r="AC36" s="2" t="str">
-        <f t="shared" ref="AC36:AC67" si="49">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=22,MATCH($D36,$H$3:$AI$3,0)&gt;=22),1,""),"")</f>
+        <f t="shared" ref="AC36:AC67" si="49">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=22,MATCH($E36,$H$3:$AI$3,0)&gt;=22),1,""),"")</f>
         <v/>
       </c>
       <c r="AD36" s="2" t="str">
-        <f t="shared" ref="AD36:AD67" si="50">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=23,MATCH($D36,$H$3:$AI$3,0)&gt;=23),1,""),"")</f>
+        <f t="shared" ref="AD36:AD67" si="50">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=23,MATCH($E36,$H$3:$AI$3,0)&gt;=23),1,""),"")</f>
         <v/>
       </c>
       <c r="AE36" s="2" t="str">
-        <f t="shared" ref="AE36:AE67" si="51">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=24,MATCH($D36,$H$3:$AI$3,0)&gt;=24),1,""),"")</f>
+        <f t="shared" ref="AE36:AE67" si="51">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=24,MATCH($E36,$H$3:$AI$3,0)&gt;=24),1,""),"")</f>
         <v/>
       </c>
       <c r="AF36" s="2" t="str">
-        <f t="shared" ref="AF36:AF67" si="52">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=25,MATCH($D36,$H$3:$AI$3,0)&gt;=25),1,""),"")</f>
+        <f t="shared" ref="AF36:AF67" si="52">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=25,MATCH($E36,$H$3:$AI$3,0)&gt;=25),1,""),"")</f>
         <v/>
       </c>
       <c r="AG36" s="2" t="str">
-        <f t="shared" ref="AG36:AG67" si="53">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=26,MATCH($D36,$H$3:$AI$3,0)&gt;=26),1,""),"")</f>
+        <f t="shared" ref="AG36:AG67" si="53">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=26,MATCH($E36,$H$3:$AI$3,0)&gt;=26),1,""),"")</f>
         <v/>
       </c>
       <c r="AH36" s="2" t="str">
-        <f t="shared" ref="AH36:AH67" si="54">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=27,MATCH($D36,$H$3:$AI$3,0)&gt;=27),1,""),"")</f>
+        <f t="shared" ref="AH36:AH67" si="54">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=27,MATCH($E36,$H$3:$AI$3,0)&gt;=27),1,""),"")</f>
         <v/>
       </c>
       <c r="AI36" s="14" t="str">
-        <f t="shared" ref="AI36:AI67" si="55">IFERROR(IF(AND(MATCH($C36,$H$3:$AI$3,0)&lt;=28,MATCH($D36,$H$3:$AI$3,0)&gt;=28),1,""),"")</f>
+        <f t="shared" ref="AI36:AI67" si="55">IFERROR(IF(AND(MATCH($D36,$H$3:$AI$3,0)&lt;=28,MATCH($E36,$H$3:$AI$3,0)&gt;=28),1,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="37" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="19"/>
-      <c r="B37" s="20"/>
+      <c r="B37" s="16"/>
       <c r="C37" s="20"/>
       <c r="D37" s="20"/>
-      <c r="E37" s="21" t="b">
+      <c r="E37" s="20"/>
+      <c r="F37" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F37" s="19"/>
-      <c r="G37" s="16"/>
+      <c r="G37" s="19"/>
       <c r="H37" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -5371,14 +5371,14 @@
     </row>
     <row r="38" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="19"/>
-      <c r="B38" s="20"/>
+      <c r="B38" s="16"/>
       <c r="C38" s="20"/>
       <c r="D38" s="20"/>
-      <c r="E38" s="21" t="b">
+      <c r="E38" s="20"/>
+      <c r="F38" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F38" s="19"/>
-      <c r="G38" s="16"/>
+      <c r="G38" s="19"/>
       <c r="H38" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -5494,14 +5494,14 @@
     </row>
     <row r="39" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="19"/>
-      <c r="B39" s="20"/>
+      <c r="B39" s="16"/>
       <c r="C39" s="20"/>
       <c r="D39" s="20"/>
-      <c r="E39" s="21" t="b">
+      <c r="E39" s="20"/>
+      <c r="F39" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F39" s="19"/>
-      <c r="G39" s="16"/>
+      <c r="G39" s="19"/>
       <c r="H39" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -5617,14 +5617,14 @@
     </row>
     <row r="40" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="19"/>
-      <c r="B40" s="20"/>
+      <c r="B40" s="16"/>
       <c r="C40" s="20"/>
       <c r="D40" s="20"/>
-      <c r="E40" s="21" t="b">
+      <c r="E40" s="20"/>
+      <c r="F40" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F40" s="19"/>
-      <c r="G40" s="16"/>
+      <c r="G40" s="19"/>
       <c r="H40" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -5740,14 +5740,14 @@
     </row>
     <row r="41" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="19"/>
-      <c r="B41" s="20"/>
+      <c r="B41" s="16"/>
       <c r="C41" s="20"/>
       <c r="D41" s="20"/>
-      <c r="E41" s="21" t="b">
+      <c r="E41" s="20"/>
+      <c r="F41" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F41" s="19"/>
-      <c r="G41" s="16"/>
+      <c r="G41" s="19"/>
       <c r="H41" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -5863,14 +5863,14 @@
     </row>
     <row r="42" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="19"/>
-      <c r="B42" s="20"/>
+      <c r="B42" s="16"/>
       <c r="C42" s="20"/>
       <c r="D42" s="20"/>
-      <c r="E42" s="21" t="b">
+      <c r="E42" s="20"/>
+      <c r="F42" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F42" s="19"/>
-      <c r="G42" s="16"/>
+      <c r="G42" s="19"/>
       <c r="H42" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -5986,14 +5986,14 @@
     </row>
     <row r="43" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="19"/>
-      <c r="B43" s="20"/>
+      <c r="B43" s="16"/>
       <c r="C43" s="20"/>
       <c r="D43" s="20"/>
-      <c r="E43" s="21" t="b">
+      <c r="E43" s="20"/>
+      <c r="F43" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F43" s="19"/>
-      <c r="G43" s="16"/>
+      <c r="G43" s="19"/>
       <c r="H43" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -6109,14 +6109,14 @@
     </row>
     <row r="44" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="19"/>
-      <c r="B44" s="20"/>
+      <c r="B44" s="16"/>
       <c r="C44" s="20"/>
       <c r="D44" s="20"/>
-      <c r="E44" s="21" t="b">
+      <c r="E44" s="20"/>
+      <c r="F44" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F44" s="19"/>
-      <c r="G44" s="16"/>
+      <c r="G44" s="19"/>
       <c r="H44" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -6232,14 +6232,14 @@
     </row>
     <row r="45" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="19"/>
-      <c r="B45" s="20"/>
+      <c r="B45" s="16"/>
       <c r="C45" s="20"/>
       <c r="D45" s="20"/>
-      <c r="E45" s="21" t="b">
+      <c r="E45" s="20"/>
+      <c r="F45" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F45" s="19"/>
-      <c r="G45" s="16"/>
+      <c r="G45" s="19"/>
       <c r="H45" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -6355,14 +6355,14 @@
     </row>
     <row r="46" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="19"/>
-      <c r="B46" s="20"/>
+      <c r="B46" s="16"/>
       <c r="C46" s="20"/>
       <c r="D46" s="20"/>
-      <c r="E46" s="21" t="b">
+      <c r="E46" s="20"/>
+      <c r="F46" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F46" s="19"/>
-      <c r="G46" s="16"/>
+      <c r="G46" s="19"/>
       <c r="H46" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -6478,14 +6478,14 @@
     </row>
     <row r="47" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="19"/>
-      <c r="B47" s="20"/>
+      <c r="B47" s="16"/>
       <c r="C47" s="20"/>
       <c r="D47" s="20"/>
-      <c r="E47" s="21" t="b">
+      <c r="E47" s="20"/>
+      <c r="F47" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F47" s="19"/>
-      <c r="G47" s="16"/>
+      <c r="G47" s="19"/>
       <c r="H47" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -6601,14 +6601,14 @@
     </row>
     <row r="48" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="19"/>
-      <c r="B48" s="20"/>
+      <c r="B48" s="16"/>
       <c r="C48" s="20"/>
       <c r="D48" s="20"/>
-      <c r="E48" s="21" t="b">
+      <c r="E48" s="20"/>
+      <c r="F48" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F48" s="19"/>
-      <c r="G48" s="16"/>
+      <c r="G48" s="19"/>
       <c r="H48" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -6724,14 +6724,14 @@
     </row>
     <row r="49" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="19"/>
-      <c r="B49" s="20"/>
+      <c r="B49" s="16"/>
       <c r="C49" s="20"/>
       <c r="D49" s="20"/>
-      <c r="E49" s="21" t="b">
+      <c r="E49" s="20"/>
+      <c r="F49" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F49" s="19"/>
-      <c r="G49" s="16"/>
+      <c r="G49" s="19"/>
       <c r="H49" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -6847,14 +6847,14 @@
     </row>
     <row r="50" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="19"/>
-      <c r="B50" s="20"/>
+      <c r="B50" s="16"/>
       <c r="C50" s="20"/>
       <c r="D50" s="20"/>
-      <c r="E50" s="21" t="b">
+      <c r="E50" s="20"/>
+      <c r="F50" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F50" s="19"/>
-      <c r="G50" s="16"/>
+      <c r="G50" s="19"/>
       <c r="H50" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -6970,14 +6970,14 @@
     </row>
     <row r="51" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="19"/>
-      <c r="B51" s="20"/>
+      <c r="B51" s="16"/>
       <c r="C51" s="20"/>
       <c r="D51" s="20"/>
-      <c r="E51" s="21" t="b">
+      <c r="E51" s="20"/>
+      <c r="F51" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F51" s="19"/>
-      <c r="G51" s="16"/>
+      <c r="G51" s="19"/>
       <c r="H51" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -7093,14 +7093,14 @@
     </row>
     <row r="52" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="19"/>
-      <c r="B52" s="20"/>
+      <c r="B52" s="16"/>
       <c r="C52" s="20"/>
       <c r="D52" s="20"/>
-      <c r="E52" s="21" t="b">
+      <c r="E52" s="20"/>
+      <c r="F52" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F52" s="19"/>
-      <c r="G52" s="16"/>
+      <c r="G52" s="19"/>
       <c r="H52" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -7216,14 +7216,14 @@
     </row>
     <row r="53" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="19"/>
-      <c r="B53" s="20"/>
+      <c r="B53" s="16"/>
       <c r="C53" s="20"/>
       <c r="D53" s="20"/>
-      <c r="E53" s="21" t="b">
+      <c r="E53" s="20"/>
+      <c r="F53" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F53" s="19"/>
-      <c r="G53" s="16"/>
+      <c r="G53" s="19"/>
       <c r="H53" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -7339,14 +7339,14 @@
     </row>
     <row r="54" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="19"/>
-      <c r="B54" s="20"/>
+      <c r="B54" s="16"/>
       <c r="C54" s="20"/>
       <c r="D54" s="20"/>
-      <c r="E54" s="21" t="b">
+      <c r="E54" s="20"/>
+      <c r="F54" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F54" s="19"/>
-      <c r="G54" s="16"/>
+      <c r="G54" s="19"/>
       <c r="H54" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -7462,14 +7462,14 @@
     </row>
     <row r="55" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="19"/>
-      <c r="B55" s="20"/>
+      <c r="B55" s="16"/>
       <c r="C55" s="20"/>
       <c r="D55" s="20"/>
-      <c r="E55" s="21" t="b">
+      <c r="E55" s="20"/>
+      <c r="F55" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F55" s="19"/>
-      <c r="G55" s="16"/>
+      <c r="G55" s="19"/>
       <c r="H55" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -7585,14 +7585,14 @@
     </row>
     <row r="56" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="19"/>
-      <c r="B56" s="20"/>
+      <c r="B56" s="16"/>
       <c r="C56" s="20"/>
       <c r="D56" s="20"/>
-      <c r="E56" s="21" t="b">
+      <c r="E56" s="20"/>
+      <c r="F56" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F56" s="19"/>
-      <c r="G56" s="16"/>
+      <c r="G56" s="19"/>
       <c r="H56" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -7708,14 +7708,14 @@
     </row>
     <row r="57" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="19"/>
-      <c r="B57" s="20"/>
+      <c r="B57" s="16"/>
       <c r="C57" s="20"/>
       <c r="D57" s="20"/>
-      <c r="E57" s="21" t="b">
+      <c r="E57" s="20"/>
+      <c r="F57" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F57" s="19"/>
-      <c r="G57" s="16"/>
+      <c r="G57" s="19"/>
       <c r="H57" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -7831,14 +7831,14 @@
     </row>
     <row r="58" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="19"/>
-      <c r="B58" s="20"/>
+      <c r="B58" s="16"/>
       <c r="C58" s="20"/>
       <c r="D58" s="20"/>
-      <c r="E58" s="21" t="b">
+      <c r="E58" s="20"/>
+      <c r="F58" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F58" s="19"/>
-      <c r="G58" s="16"/>
+      <c r="G58" s="19"/>
       <c r="H58" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -7954,14 +7954,14 @@
     </row>
     <row r="59" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="19"/>
-      <c r="B59" s="20"/>
+      <c r="B59" s="16"/>
       <c r="C59" s="20"/>
       <c r="D59" s="20"/>
-      <c r="E59" s="21" t="b">
+      <c r="E59" s="20"/>
+      <c r="F59" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F59" s="19"/>
-      <c r="G59" s="16"/>
+      <c r="G59" s="19"/>
       <c r="H59" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -8077,14 +8077,14 @@
     </row>
     <row r="60" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
-      <c r="B60" s="20"/>
+      <c r="B60" s="16"/>
       <c r="C60" s="20"/>
       <c r="D60" s="20"/>
-      <c r="E60" s="21" t="b">
+      <c r="E60" s="20"/>
+      <c r="F60" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F60" s="19"/>
-      <c r="G60" s="16"/>
+      <c r="G60" s="19"/>
       <c r="H60" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -8200,14 +8200,14 @@
     </row>
     <row r="61" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="19"/>
-      <c r="B61" s="20"/>
+      <c r="B61" s="16"/>
       <c r="C61" s="20"/>
       <c r="D61" s="20"/>
-      <c r="E61" s="21" t="b">
+      <c r="E61" s="20"/>
+      <c r="F61" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F61" s="19"/>
-      <c r="G61" s="16"/>
+      <c r="G61" s="19"/>
       <c r="H61" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -8323,14 +8323,14 @@
     </row>
     <row r="62" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
-      <c r="B62" s="20"/>
+      <c r="B62" s="16"/>
       <c r="C62" s="20"/>
       <c r="D62" s="20"/>
-      <c r="E62" s="21" t="b">
+      <c r="E62" s="20"/>
+      <c r="F62" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F62" s="19"/>
-      <c r="G62" s="16"/>
+      <c r="G62" s="19"/>
       <c r="H62" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -8446,14 +8446,14 @@
     </row>
     <row r="63" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="19"/>
-      <c r="B63" s="20"/>
+      <c r="B63" s="16"/>
       <c r="C63" s="20"/>
       <c r="D63" s="20"/>
-      <c r="E63" s="21" t="b">
+      <c r="E63" s="20"/>
+      <c r="F63" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F63" s="19"/>
-      <c r="G63" s="16"/>
+      <c r="G63" s="19"/>
       <c r="H63" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -8569,14 +8569,14 @@
     </row>
     <row r="64" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="19"/>
-      <c r="B64" s="20"/>
+      <c r="B64" s="16"/>
       <c r="C64" s="20"/>
       <c r="D64" s="20"/>
-      <c r="E64" s="21" t="b">
+      <c r="E64" s="20"/>
+      <c r="F64" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F64" s="19"/>
-      <c r="G64" s="16"/>
+      <c r="G64" s="19"/>
       <c r="H64" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -8692,14 +8692,14 @@
     </row>
     <row r="65" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="19"/>
-      <c r="B65" s="20"/>
+      <c r="B65" s="16"/>
       <c r="C65" s="20"/>
       <c r="D65" s="20"/>
-      <c r="E65" s="21" t="b">
+      <c r="E65" s="20"/>
+      <c r="F65" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F65" s="19"/>
-      <c r="G65" s="16"/>
+      <c r="G65" s="19"/>
       <c r="H65" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -8815,14 +8815,14 @@
     </row>
     <row r="66" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="19"/>
-      <c r="B66" s="20"/>
+      <c r="B66" s="16"/>
       <c r="C66" s="20"/>
       <c r="D66" s="20"/>
-      <c r="E66" s="21" t="b">
+      <c r="E66" s="20"/>
+      <c r="F66" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F66" s="19"/>
-      <c r="G66" s="16"/>
+      <c r="G66" s="19"/>
       <c r="H66" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -8938,14 +8938,14 @@
     </row>
     <row r="67" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="19"/>
-      <c r="B67" s="20"/>
+      <c r="B67" s="16"/>
       <c r="C67" s="20"/>
       <c r="D67" s="20"/>
-      <c r="E67" s="21" t="b">
+      <c r="E67" s="20"/>
+      <c r="F67" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F67" s="19"/>
-      <c r="G67" s="16"/>
+      <c r="G67" s="19"/>
       <c r="H67" s="1" t="str">
         <f t="shared" si="28"/>
         <v/>
@@ -9061,137 +9061,137 @@
     </row>
     <row r="68" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="19"/>
-      <c r="B68" s="20"/>
+      <c r="B68" s="16"/>
       <c r="C68" s="20"/>
       <c r="D68" s="20"/>
-      <c r="E68" s="21" t="b">
+      <c r="E68" s="20"/>
+      <c r="F68" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F68" s="19"/>
-      <c r="G68" s="16"/>
+      <c r="G68" s="19"/>
       <c r="H68" s="1" t="str">
-        <f t="shared" ref="H68:H99" si="56">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=1,MATCH($D68,$H$3:$AI$3,0)&gt;=1),1,""),"")</f>
+        <f t="shared" ref="H68:H99" si="56">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=1,MATCH($E68,$H$3:$AI$3,0)&gt;=1),1,""),"")</f>
         <v/>
       </c>
       <c r="I68" s="2" t="str">
-        <f t="shared" ref="I68:I99" si="57">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=2,MATCH($D68,$H$3:$AI$3,0)&gt;=2),1,""),"")</f>
+        <f t="shared" ref="I68:I99" si="57">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=2,MATCH($E68,$H$3:$AI$3,0)&gt;=2),1,""),"")</f>
         <v/>
       </c>
       <c r="J68" s="2" t="str">
-        <f t="shared" ref="J68:J99" si="58">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=3,MATCH($D68,$H$3:$AI$3,0)&gt;=3),1,""),"")</f>
+        <f t="shared" ref="J68:J99" si="58">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=3,MATCH($E68,$H$3:$AI$3,0)&gt;=3),1,""),"")</f>
         <v/>
       </c>
       <c r="K68" s="2" t="str">
-        <f t="shared" ref="K68:K99" si="59">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=4,MATCH($D68,$H$3:$AI$3,0)&gt;=4),1,""),"")</f>
+        <f t="shared" ref="K68:K99" si="59">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=4,MATCH($E68,$H$3:$AI$3,0)&gt;=4),1,""),"")</f>
         <v/>
       </c>
       <c r="L68" s="2" t="str">
-        <f t="shared" ref="L68:L99" si="60">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=5,MATCH($D68,$H$3:$AI$3,0)&gt;=5),1,""),"")</f>
+        <f t="shared" ref="L68:L99" si="60">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=5,MATCH($E68,$H$3:$AI$3,0)&gt;=5),1,""),"")</f>
         <v/>
       </c>
       <c r="M68" s="2" t="str">
-        <f t="shared" ref="M68:M99" si="61">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=6,MATCH($D68,$H$3:$AI$3,0)&gt;=6),1,""),"")</f>
+        <f t="shared" ref="M68:M99" si="61">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=6,MATCH($E68,$H$3:$AI$3,0)&gt;=6),1,""),"")</f>
         <v/>
       </c>
       <c r="N68" s="2" t="str">
-        <f t="shared" ref="N68:N99" si="62">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=7,MATCH($D68,$H$3:$AI$3,0)&gt;=7),1,""),"")</f>
+        <f t="shared" ref="N68:N99" si="62">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=7,MATCH($E68,$H$3:$AI$3,0)&gt;=7),1,""),"")</f>
         <v/>
       </c>
       <c r="O68" s="2" t="str">
-        <f t="shared" ref="O68:O99" si="63">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=8,MATCH($D68,$H$3:$AI$3,0)&gt;=8),1,""),"")</f>
+        <f t="shared" ref="O68:O99" si="63">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=8,MATCH($E68,$H$3:$AI$3,0)&gt;=8),1,""),"")</f>
         <v/>
       </c>
       <c r="P68" s="2" t="str">
-        <f t="shared" ref="P68:P99" si="64">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=9,MATCH($D68,$H$3:$AI$3,0)&gt;=9),1,""),"")</f>
+        <f t="shared" ref="P68:P99" si="64">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=9,MATCH($E68,$H$3:$AI$3,0)&gt;=9),1,""),"")</f>
         <v/>
       </c>
       <c r="Q68" s="2" t="str">
-        <f t="shared" ref="Q68:Q99" si="65">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=10,MATCH($D68,$H$3:$AI$3,0)&gt;=10),1,""),"")</f>
+        <f t="shared" ref="Q68:Q99" si="65">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=10,MATCH($E68,$H$3:$AI$3,0)&gt;=10),1,""),"")</f>
         <v/>
       </c>
       <c r="R68" s="2" t="str">
-        <f t="shared" ref="R68:R99" si="66">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=11,MATCH($D68,$H$3:$AI$3,0)&gt;=11),1,""),"")</f>
+        <f t="shared" ref="R68:R99" si="66">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=11,MATCH($E68,$H$3:$AI$3,0)&gt;=11),1,""),"")</f>
         <v/>
       </c>
       <c r="S68" s="2" t="str">
-        <f t="shared" ref="S68:S99" si="67">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=12,MATCH($D68,$H$3:$AI$3,0)&gt;=12),1,""),"")</f>
+        <f t="shared" ref="S68:S99" si="67">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=12,MATCH($E68,$H$3:$AI$3,0)&gt;=12),1,""),"")</f>
         <v/>
       </c>
       <c r="T68" s="2" t="str">
-        <f t="shared" ref="T68:T99" si="68">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=13,MATCH($D68,$H$3:$AI$3,0)&gt;=13),1,""),"")</f>
+        <f t="shared" ref="T68:T99" si="68">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=13,MATCH($E68,$H$3:$AI$3,0)&gt;=13),1,""),"")</f>
         <v/>
       </c>
       <c r="U68" s="2" t="str">
-        <f t="shared" ref="U68:U99" si="69">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=14,MATCH($D68,$H$3:$AI$3,0)&gt;=14),1,""),"")</f>
+        <f t="shared" ref="U68:U99" si="69">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=14,MATCH($E68,$H$3:$AI$3,0)&gt;=14),1,""),"")</f>
         <v/>
       </c>
       <c r="V68" s="2" t="str">
-        <f t="shared" ref="V68:V99" si="70">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=15,MATCH($D68,$H$3:$AI$3,0)&gt;=15),1,""),"")</f>
+        <f t="shared" ref="V68:V99" si="70">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=15,MATCH($E68,$H$3:$AI$3,0)&gt;=15),1,""),"")</f>
         <v/>
       </c>
       <c r="W68" s="2" t="str">
-        <f t="shared" ref="W68:W99" si="71">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=16,MATCH($D68,$H$3:$AI$3,0)&gt;=16),1,""),"")</f>
+        <f t="shared" ref="W68:W99" si="71">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=16,MATCH($E68,$H$3:$AI$3,0)&gt;=16),1,""),"")</f>
         <v/>
       </c>
       <c r="X68" s="2" t="str">
-        <f t="shared" ref="X68:X99" si="72">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=17,MATCH($D68,$H$3:$AI$3,0)&gt;=17),1,""),"")</f>
+        <f t="shared" ref="X68:X99" si="72">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=17,MATCH($E68,$H$3:$AI$3,0)&gt;=17),1,""),"")</f>
         <v/>
       </c>
       <c r="Y68" s="2" t="str">
-        <f t="shared" ref="Y68:Y99" si="73">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=18,MATCH($D68,$H$3:$AI$3,0)&gt;=18),1,""),"")</f>
+        <f t="shared" ref="Y68:Y99" si="73">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=18,MATCH($E68,$H$3:$AI$3,0)&gt;=18),1,""),"")</f>
         <v/>
       </c>
       <c r="Z68" s="2" t="str">
-        <f t="shared" ref="Z68:Z99" si="74">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=19,MATCH($D68,$H$3:$AI$3,0)&gt;=19),1,""),"")</f>
+        <f t="shared" ref="Z68:Z99" si="74">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=19,MATCH($E68,$H$3:$AI$3,0)&gt;=19),1,""),"")</f>
         <v/>
       </c>
       <c r="AA68" s="2" t="str">
-        <f t="shared" ref="AA68:AA99" si="75">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=20,MATCH($D68,$H$3:$AI$3,0)&gt;=20),1,""),"")</f>
+        <f t="shared" ref="AA68:AA99" si="75">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=20,MATCH($E68,$H$3:$AI$3,0)&gt;=20),1,""),"")</f>
         <v/>
       </c>
       <c r="AB68" s="2" t="str">
-        <f t="shared" ref="AB68:AB99" si="76">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=21,MATCH($D68,$H$3:$AI$3,0)&gt;=21),1,""),"")</f>
+        <f t="shared" ref="AB68:AB99" si="76">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=21,MATCH($E68,$H$3:$AI$3,0)&gt;=21),1,""),"")</f>
         <v/>
       </c>
       <c r="AC68" s="2" t="str">
-        <f t="shared" ref="AC68:AC99" si="77">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=22,MATCH($D68,$H$3:$AI$3,0)&gt;=22),1,""),"")</f>
+        <f t="shared" ref="AC68:AC99" si="77">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=22,MATCH($E68,$H$3:$AI$3,0)&gt;=22),1,""),"")</f>
         <v/>
       </c>
       <c r="AD68" s="2" t="str">
-        <f t="shared" ref="AD68:AD99" si="78">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=23,MATCH($D68,$H$3:$AI$3,0)&gt;=23),1,""),"")</f>
+        <f t="shared" ref="AD68:AD99" si="78">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=23,MATCH($E68,$H$3:$AI$3,0)&gt;=23),1,""),"")</f>
         <v/>
       </c>
       <c r="AE68" s="2" t="str">
-        <f t="shared" ref="AE68:AE99" si="79">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=24,MATCH($D68,$H$3:$AI$3,0)&gt;=24),1,""),"")</f>
+        <f t="shared" ref="AE68:AE99" si="79">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=24,MATCH($E68,$H$3:$AI$3,0)&gt;=24),1,""),"")</f>
         <v/>
       </c>
       <c r="AF68" s="2" t="str">
-        <f t="shared" ref="AF68:AF99" si="80">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=25,MATCH($D68,$H$3:$AI$3,0)&gt;=25),1,""),"")</f>
+        <f t="shared" ref="AF68:AF99" si="80">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=25,MATCH($E68,$H$3:$AI$3,0)&gt;=25),1,""),"")</f>
         <v/>
       </c>
       <c r="AG68" s="2" t="str">
-        <f t="shared" ref="AG68:AG99" si="81">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=26,MATCH($D68,$H$3:$AI$3,0)&gt;=26),1,""),"")</f>
+        <f t="shared" ref="AG68:AG99" si="81">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=26,MATCH($E68,$H$3:$AI$3,0)&gt;=26),1,""),"")</f>
         <v/>
       </c>
       <c r="AH68" s="2" t="str">
-        <f t="shared" ref="AH68:AH99" si="82">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=27,MATCH($D68,$H$3:$AI$3,0)&gt;=27),1,""),"")</f>
+        <f t="shared" ref="AH68:AH99" si="82">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=27,MATCH($E68,$H$3:$AI$3,0)&gt;=27),1,""),"")</f>
         <v/>
       </c>
       <c r="AI68" s="14" t="str">
-        <f t="shared" ref="AI68:AI99" si="83">IFERROR(IF(AND(MATCH($C68,$H$3:$AI$3,0)&lt;=28,MATCH($D68,$H$3:$AI$3,0)&gt;=28),1,""),"")</f>
+        <f t="shared" ref="AI68:AI99" si="83">IFERROR(IF(AND(MATCH($D68,$H$3:$AI$3,0)&lt;=28,MATCH($E68,$H$3:$AI$3,0)&gt;=28),1,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="69" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="19"/>
-      <c r="B69" s="20"/>
+      <c r="B69" s="16"/>
       <c r="C69" s="20"/>
       <c r="D69" s="20"/>
-      <c r="E69" s="21" t="b">
+      <c r="E69" s="20"/>
+      <c r="F69" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F69" s="19"/>
-      <c r="G69" s="16"/>
+      <c r="G69" s="19"/>
       <c r="H69" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -9307,14 +9307,14 @@
     </row>
     <row r="70" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="19"/>
-      <c r="B70" s="20"/>
+      <c r="B70" s="16"/>
       <c r="C70" s="20"/>
       <c r="D70" s="20"/>
-      <c r="E70" s="21" t="b">
+      <c r="E70" s="20"/>
+      <c r="F70" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F70" s="19"/>
-      <c r="G70" s="16"/>
+      <c r="G70" s="19"/>
       <c r="H70" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -9430,14 +9430,14 @@
     </row>
     <row r="71" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="19"/>
-      <c r="B71" s="20"/>
+      <c r="B71" s="16"/>
       <c r="C71" s="20"/>
       <c r="D71" s="20"/>
-      <c r="E71" s="21" t="b">
+      <c r="E71" s="20"/>
+      <c r="F71" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F71" s="19"/>
-      <c r="G71" s="16"/>
+      <c r="G71" s="19"/>
       <c r="H71" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -9553,14 +9553,14 @@
     </row>
     <row r="72" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="19"/>
-      <c r="B72" s="20"/>
+      <c r="B72" s="16"/>
       <c r="C72" s="20"/>
       <c r="D72" s="20"/>
-      <c r="E72" s="21" t="b">
+      <c r="E72" s="20"/>
+      <c r="F72" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F72" s="19"/>
-      <c r="G72" s="16"/>
+      <c r="G72" s="19"/>
       <c r="H72" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -9676,14 +9676,14 @@
     </row>
     <row r="73" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="19"/>
-      <c r="B73" s="20"/>
+      <c r="B73" s="16"/>
       <c r="C73" s="20"/>
       <c r="D73" s="20"/>
-      <c r="E73" s="21" t="b">
+      <c r="E73" s="20"/>
+      <c r="F73" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F73" s="19"/>
-      <c r="G73" s="16"/>
+      <c r="G73" s="19"/>
       <c r="H73" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -9799,14 +9799,14 @@
     </row>
     <row r="74" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="19"/>
-      <c r="B74" s="20"/>
+      <c r="B74" s="16"/>
       <c r="C74" s="20"/>
       <c r="D74" s="20"/>
-      <c r="E74" s="21" t="b">
+      <c r="E74" s="20"/>
+      <c r="F74" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F74" s="19"/>
-      <c r="G74" s="16"/>
+      <c r="G74" s="19"/>
       <c r="H74" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -9922,14 +9922,14 @@
     </row>
     <row r="75" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="19"/>
-      <c r="B75" s="20"/>
+      <c r="B75" s="16"/>
       <c r="C75" s="20"/>
       <c r="D75" s="20"/>
-      <c r="E75" s="21" t="b">
+      <c r="E75" s="20"/>
+      <c r="F75" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F75" s="19"/>
-      <c r="G75" s="16"/>
+      <c r="G75" s="19"/>
       <c r="H75" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -10045,14 +10045,14 @@
     </row>
     <row r="76" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="19"/>
-      <c r="B76" s="20"/>
+      <c r="B76" s="16"/>
       <c r="C76" s="20"/>
       <c r="D76" s="20"/>
-      <c r="E76" s="21" t="b">
+      <c r="E76" s="20"/>
+      <c r="F76" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F76" s="19"/>
-      <c r="G76" s="16"/>
+      <c r="G76" s="19"/>
       <c r="H76" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -10168,14 +10168,14 @@
     </row>
     <row r="77" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="19"/>
-      <c r="B77" s="20"/>
+      <c r="B77" s="16"/>
       <c r="C77" s="20"/>
       <c r="D77" s="20"/>
-      <c r="E77" s="21" t="b">
+      <c r="E77" s="20"/>
+      <c r="F77" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F77" s="19"/>
-      <c r="G77" s="16"/>
+      <c r="G77" s="19"/>
       <c r="H77" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -10291,14 +10291,14 @@
     </row>
     <row r="78" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="19"/>
-      <c r="B78" s="20"/>
+      <c r="B78" s="16"/>
       <c r="C78" s="20"/>
       <c r="D78" s="20"/>
-      <c r="E78" s="21" t="b">
+      <c r="E78" s="20"/>
+      <c r="F78" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F78" s="19"/>
-      <c r="G78" s="16"/>
+      <c r="G78" s="19"/>
       <c r="H78" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -10414,14 +10414,14 @@
     </row>
     <row r="79" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="19"/>
-      <c r="B79" s="20"/>
+      <c r="B79" s="16"/>
       <c r="C79" s="20"/>
       <c r="D79" s="20"/>
-      <c r="E79" s="21" t="b">
+      <c r="E79" s="20"/>
+      <c r="F79" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F79" s="19"/>
-      <c r="G79" s="16"/>
+      <c r="G79" s="19"/>
       <c r="H79" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -10537,14 +10537,14 @@
     </row>
     <row r="80" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="19"/>
-      <c r="B80" s="20"/>
+      <c r="B80" s="16"/>
       <c r="C80" s="20"/>
       <c r="D80" s="20"/>
-      <c r="E80" s="21" t="b">
+      <c r="E80" s="20"/>
+      <c r="F80" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F80" s="19"/>
-      <c r="G80" s="16"/>
+      <c r="G80" s="19"/>
       <c r="H80" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -10660,14 +10660,14 @@
     </row>
     <row r="81" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="19"/>
-      <c r="B81" s="20"/>
+      <c r="B81" s="16"/>
       <c r="C81" s="20"/>
       <c r="D81" s="20"/>
-      <c r="E81" s="21" t="b">
+      <c r="E81" s="20"/>
+      <c r="F81" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F81" s="19"/>
-      <c r="G81" s="16"/>
+      <c r="G81" s="19"/>
       <c r="H81" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -10783,14 +10783,14 @@
     </row>
     <row r="82" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="19"/>
-      <c r="B82" s="20"/>
+      <c r="B82" s="16"/>
       <c r="C82" s="20"/>
       <c r="D82" s="20"/>
-      <c r="E82" s="21" t="b">
+      <c r="E82" s="20"/>
+      <c r="F82" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F82" s="19"/>
-      <c r="G82" s="16"/>
+      <c r="G82" s="19"/>
       <c r="H82" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -10906,14 +10906,14 @@
     </row>
     <row r="83" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="19"/>
-      <c r="B83" s="20"/>
+      <c r="B83" s="16"/>
       <c r="C83" s="20"/>
       <c r="D83" s="20"/>
-      <c r="E83" s="21" t="b">
+      <c r="E83" s="20"/>
+      <c r="F83" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F83" s="19"/>
-      <c r="G83" s="16"/>
+      <c r="G83" s="19"/>
       <c r="H83" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -11029,14 +11029,14 @@
     </row>
     <row r="84" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="19"/>
-      <c r="B84" s="20"/>
+      <c r="B84" s="16"/>
       <c r="C84" s="20"/>
       <c r="D84" s="20"/>
-      <c r="E84" s="21" t="b">
+      <c r="E84" s="20"/>
+      <c r="F84" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F84" s="19"/>
-      <c r="G84" s="16"/>
+      <c r="G84" s="19"/>
       <c r="H84" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -11152,14 +11152,14 @@
     </row>
     <row r="85" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="19"/>
-      <c r="B85" s="20"/>
+      <c r="B85" s="16"/>
       <c r="C85" s="20"/>
       <c r="D85" s="20"/>
-      <c r="E85" s="21" t="b">
+      <c r="E85" s="20"/>
+      <c r="F85" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F85" s="19"/>
-      <c r="G85" s="16"/>
+      <c r="G85" s="19"/>
       <c r="H85" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -11275,14 +11275,14 @@
     </row>
     <row r="86" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="19"/>
-      <c r="B86" s="20"/>
+      <c r="B86" s="16"/>
       <c r="C86" s="20"/>
       <c r="D86" s="20"/>
-      <c r="E86" s="21" t="b">
+      <c r="E86" s="20"/>
+      <c r="F86" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F86" s="19"/>
-      <c r="G86" s="16"/>
+      <c r="G86" s="19"/>
       <c r="H86" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -11398,14 +11398,14 @@
     </row>
     <row r="87" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="19"/>
-      <c r="B87" s="20"/>
+      <c r="B87" s="16"/>
       <c r="C87" s="20"/>
       <c r="D87" s="20"/>
-      <c r="E87" s="21" t="b">
+      <c r="E87" s="20"/>
+      <c r="F87" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F87" s="19"/>
-      <c r="G87" s="16"/>
+      <c r="G87" s="19"/>
       <c r="H87" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -11521,14 +11521,14 @@
     </row>
     <row r="88" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="19"/>
-      <c r="B88" s="20"/>
+      <c r="B88" s="16"/>
       <c r="C88" s="20"/>
       <c r="D88" s="20"/>
-      <c r="E88" s="21" t="b">
+      <c r="E88" s="20"/>
+      <c r="F88" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F88" s="19"/>
-      <c r="G88" s="16"/>
+      <c r="G88" s="19"/>
       <c r="H88" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -11644,14 +11644,14 @@
     </row>
     <row r="89" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="19"/>
-      <c r="B89" s="20"/>
+      <c r="B89" s="16"/>
       <c r="C89" s="20"/>
       <c r="D89" s="20"/>
-      <c r="E89" s="21" t="b">
+      <c r="E89" s="20"/>
+      <c r="F89" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F89" s="19"/>
-      <c r="G89" s="16"/>
+      <c r="G89" s="19"/>
       <c r="H89" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -11767,14 +11767,14 @@
     </row>
     <row r="90" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="19"/>
-      <c r="B90" s="20"/>
+      <c r="B90" s="16"/>
       <c r="C90" s="20"/>
       <c r="D90" s="20"/>
-      <c r="E90" s="21" t="b">
+      <c r="E90" s="20"/>
+      <c r="F90" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F90" s="19"/>
-      <c r="G90" s="16"/>
+      <c r="G90" s="19"/>
       <c r="H90" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -11890,14 +11890,14 @@
     </row>
     <row r="91" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="19"/>
-      <c r="B91" s="20"/>
+      <c r="B91" s="16"/>
       <c r="C91" s="20"/>
       <c r="D91" s="20"/>
-      <c r="E91" s="21" t="b">
+      <c r="E91" s="20"/>
+      <c r="F91" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F91" s="19"/>
-      <c r="G91" s="16"/>
+      <c r="G91" s="19"/>
       <c r="H91" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -12013,14 +12013,14 @@
     </row>
     <row r="92" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="19"/>
-      <c r="B92" s="20"/>
+      <c r="B92" s="16"/>
       <c r="C92" s="20"/>
       <c r="D92" s="20"/>
-      <c r="E92" s="21" t="b">
+      <c r="E92" s="20"/>
+      <c r="F92" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F92" s="19"/>
-      <c r="G92" s="16"/>
+      <c r="G92" s="19"/>
       <c r="H92" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -12136,14 +12136,14 @@
     </row>
     <row r="93" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="19"/>
-      <c r="B93" s="20"/>
+      <c r="B93" s="16"/>
       <c r="C93" s="20"/>
       <c r="D93" s="20"/>
-      <c r="E93" s="21" t="b">
+      <c r="E93" s="20"/>
+      <c r="F93" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F93" s="19"/>
-      <c r="G93" s="16"/>
+      <c r="G93" s="19"/>
       <c r="H93" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -12259,14 +12259,14 @@
     </row>
     <row r="94" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="19"/>
-      <c r="B94" s="20"/>
+      <c r="B94" s="16"/>
       <c r="C94" s="20"/>
       <c r="D94" s="20"/>
-      <c r="E94" s="21" t="b">
+      <c r="E94" s="20"/>
+      <c r="F94" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F94" s="19"/>
-      <c r="G94" s="16"/>
+      <c r="G94" s="19"/>
       <c r="H94" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -12382,14 +12382,14 @@
     </row>
     <row r="95" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="19"/>
-      <c r="B95" s="20"/>
+      <c r="B95" s="16"/>
       <c r="C95" s="20"/>
       <c r="D95" s="20"/>
-      <c r="E95" s="21" t="b">
+      <c r="E95" s="20"/>
+      <c r="F95" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F95" s="19"/>
-      <c r="G95" s="16"/>
+      <c r="G95" s="19"/>
       <c r="H95" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -12505,14 +12505,14 @@
     </row>
     <row r="96" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="19"/>
-      <c r="B96" s="20"/>
+      <c r="B96" s="16"/>
       <c r="C96" s="20"/>
       <c r="D96" s="20"/>
-      <c r="E96" s="21" t="b">
+      <c r="E96" s="20"/>
+      <c r="F96" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F96" s="19"/>
-      <c r="G96" s="16"/>
+      <c r="G96" s="19"/>
       <c r="H96" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -12628,14 +12628,14 @@
     </row>
     <row r="97" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="19"/>
-      <c r="B97" s="20"/>
+      <c r="B97" s="16"/>
       <c r="C97" s="20"/>
       <c r="D97" s="20"/>
-      <c r="E97" s="21" t="b">
+      <c r="E97" s="20"/>
+      <c r="F97" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F97" s="19"/>
-      <c r="G97" s="16"/>
+      <c r="G97" s="19"/>
       <c r="H97" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -12751,14 +12751,14 @@
     </row>
     <row r="98" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="19"/>
-      <c r="B98" s="20"/>
+      <c r="B98" s="16"/>
       <c r="C98" s="20"/>
       <c r="D98" s="20"/>
-      <c r="E98" s="21" t="b">
+      <c r="E98" s="20"/>
+      <c r="F98" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F98" s="19"/>
-      <c r="G98" s="16"/>
+      <c r="G98" s="19"/>
       <c r="H98" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -12874,14 +12874,14 @@
     </row>
     <row r="99" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="19"/>
-      <c r="B99" s="20"/>
+      <c r="B99" s="16"/>
       <c r="C99" s="20"/>
       <c r="D99" s="20"/>
-      <c r="E99" s="21" t="b">
+      <c r="E99" s="20"/>
+      <c r="F99" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F99" s="19"/>
-      <c r="G99" s="16"/>
+      <c r="G99" s="19"/>
       <c r="H99" s="1" t="str">
         <f t="shared" si="56"/>
         <v/>
@@ -12997,137 +12997,137 @@
     </row>
     <row r="100" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="19"/>
-      <c r="B100" s="20"/>
+      <c r="B100" s="16"/>
       <c r="C100" s="20"/>
       <c r="D100" s="20"/>
-      <c r="E100" s="21" t="b">
+      <c r="E100" s="20"/>
+      <c r="F100" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F100" s="19"/>
-      <c r="G100" s="16"/>
+      <c r="G100" s="19"/>
       <c r="H100" s="1" t="str">
-        <f t="shared" ref="H100:H123" si="84">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=1,MATCH($D100,$H$3:$AI$3,0)&gt;=1),1,""),"")</f>
+        <f t="shared" ref="H100:H123" si="84">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=1,MATCH($E100,$H$3:$AI$3,0)&gt;=1),1,""),"")</f>
         <v/>
       </c>
       <c r="I100" s="2" t="str">
-        <f t="shared" ref="I100:I123" si="85">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=2,MATCH($D100,$H$3:$AI$3,0)&gt;=2),1,""),"")</f>
+        <f t="shared" ref="I100:I123" si="85">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=2,MATCH($E100,$H$3:$AI$3,0)&gt;=2),1,""),"")</f>
         <v/>
       </c>
       <c r="J100" s="2" t="str">
-        <f t="shared" ref="J100:J123" si="86">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=3,MATCH($D100,$H$3:$AI$3,0)&gt;=3),1,""),"")</f>
+        <f t="shared" ref="J100:J123" si="86">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=3,MATCH($E100,$H$3:$AI$3,0)&gt;=3),1,""),"")</f>
         <v/>
       </c>
       <c r="K100" s="2" t="str">
-        <f t="shared" ref="K100:K123" si="87">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=4,MATCH($D100,$H$3:$AI$3,0)&gt;=4),1,""),"")</f>
+        <f t="shared" ref="K100:K123" si="87">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=4,MATCH($E100,$H$3:$AI$3,0)&gt;=4),1,""),"")</f>
         <v/>
       </c>
       <c r="L100" s="2" t="str">
-        <f t="shared" ref="L100:L123" si="88">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=5,MATCH($D100,$H$3:$AI$3,0)&gt;=5),1,""),"")</f>
+        <f t="shared" ref="L100:L123" si="88">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=5,MATCH($E100,$H$3:$AI$3,0)&gt;=5),1,""),"")</f>
         <v/>
       </c>
       <c r="M100" s="2" t="str">
-        <f t="shared" ref="M100:M123" si="89">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=6,MATCH($D100,$H$3:$AI$3,0)&gt;=6),1,""),"")</f>
+        <f t="shared" ref="M100:M123" si="89">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=6,MATCH($E100,$H$3:$AI$3,0)&gt;=6),1,""),"")</f>
         <v/>
       </c>
       <c r="N100" s="2" t="str">
-        <f t="shared" ref="N100:N123" si="90">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=7,MATCH($D100,$H$3:$AI$3,0)&gt;=7),1,""),"")</f>
+        <f t="shared" ref="N100:N123" si="90">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=7,MATCH($E100,$H$3:$AI$3,0)&gt;=7),1,""),"")</f>
         <v/>
       </c>
       <c r="O100" s="2" t="str">
-        <f t="shared" ref="O100:O123" si="91">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=8,MATCH($D100,$H$3:$AI$3,0)&gt;=8),1,""),"")</f>
+        <f t="shared" ref="O100:O123" si="91">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=8,MATCH($E100,$H$3:$AI$3,0)&gt;=8),1,""),"")</f>
         <v/>
       </c>
       <c r="P100" s="2" t="str">
-        <f t="shared" ref="P100:P123" si="92">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=9,MATCH($D100,$H$3:$AI$3,0)&gt;=9),1,""),"")</f>
+        <f t="shared" ref="P100:P123" si="92">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=9,MATCH($E100,$H$3:$AI$3,0)&gt;=9),1,""),"")</f>
         <v/>
       </c>
       <c r="Q100" s="2" t="str">
-        <f t="shared" ref="Q100:Q123" si="93">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=10,MATCH($D100,$H$3:$AI$3,0)&gt;=10),1,""),"")</f>
+        <f t="shared" ref="Q100:Q123" si="93">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=10,MATCH($E100,$H$3:$AI$3,0)&gt;=10),1,""),"")</f>
         <v/>
       </c>
       <c r="R100" s="2" t="str">
-        <f t="shared" ref="R100:R123" si="94">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=11,MATCH($D100,$H$3:$AI$3,0)&gt;=11),1,""),"")</f>
+        <f t="shared" ref="R100:R123" si="94">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=11,MATCH($E100,$H$3:$AI$3,0)&gt;=11),1,""),"")</f>
         <v/>
       </c>
       <c r="S100" s="2" t="str">
-        <f t="shared" ref="S100:S123" si="95">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=12,MATCH($D100,$H$3:$AI$3,0)&gt;=12),1,""),"")</f>
+        <f t="shared" ref="S100:S123" si="95">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=12,MATCH($E100,$H$3:$AI$3,0)&gt;=12),1,""),"")</f>
         <v/>
       </c>
       <c r="T100" s="2" t="str">
-        <f t="shared" ref="T100:T123" si="96">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=13,MATCH($D100,$H$3:$AI$3,0)&gt;=13),1,""),"")</f>
+        <f t="shared" ref="T100:T123" si="96">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=13,MATCH($E100,$H$3:$AI$3,0)&gt;=13),1,""),"")</f>
         <v/>
       </c>
       <c r="U100" s="2" t="str">
-        <f t="shared" ref="U100:U123" si="97">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=14,MATCH($D100,$H$3:$AI$3,0)&gt;=14),1,""),"")</f>
+        <f t="shared" ref="U100:U123" si="97">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=14,MATCH($E100,$H$3:$AI$3,0)&gt;=14),1,""),"")</f>
         <v/>
       </c>
       <c r="V100" s="2" t="str">
-        <f t="shared" ref="V100:V123" si="98">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=15,MATCH($D100,$H$3:$AI$3,0)&gt;=15),1,""),"")</f>
+        <f t="shared" ref="V100:V123" si="98">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=15,MATCH($E100,$H$3:$AI$3,0)&gt;=15),1,""),"")</f>
         <v/>
       </c>
       <c r="W100" s="2" t="str">
-        <f t="shared" ref="W100:W123" si="99">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=16,MATCH($D100,$H$3:$AI$3,0)&gt;=16),1,""),"")</f>
+        <f t="shared" ref="W100:W123" si="99">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=16,MATCH($E100,$H$3:$AI$3,0)&gt;=16),1,""),"")</f>
         <v/>
       </c>
       <c r="X100" s="2" t="str">
-        <f t="shared" ref="X100:X123" si="100">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=17,MATCH($D100,$H$3:$AI$3,0)&gt;=17),1,""),"")</f>
+        <f t="shared" ref="X100:X123" si="100">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=17,MATCH($E100,$H$3:$AI$3,0)&gt;=17),1,""),"")</f>
         <v/>
       </c>
       <c r="Y100" s="2" t="str">
-        <f t="shared" ref="Y100:Y123" si="101">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=18,MATCH($D100,$H$3:$AI$3,0)&gt;=18),1,""),"")</f>
+        <f t="shared" ref="Y100:Y123" si="101">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=18,MATCH($E100,$H$3:$AI$3,0)&gt;=18),1,""),"")</f>
         <v/>
       </c>
       <c r="Z100" s="2" t="str">
-        <f t="shared" ref="Z100:Z123" si="102">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=19,MATCH($D100,$H$3:$AI$3,0)&gt;=19),1,""),"")</f>
+        <f t="shared" ref="Z100:Z123" si="102">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=19,MATCH($E100,$H$3:$AI$3,0)&gt;=19),1,""),"")</f>
         <v/>
       </c>
       <c r="AA100" s="2" t="str">
-        <f t="shared" ref="AA100:AA123" si="103">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=20,MATCH($D100,$H$3:$AI$3,0)&gt;=20),1,""),"")</f>
+        <f t="shared" ref="AA100:AA123" si="103">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=20,MATCH($E100,$H$3:$AI$3,0)&gt;=20),1,""),"")</f>
         <v/>
       </c>
       <c r="AB100" s="2" t="str">
-        <f t="shared" ref="AB100:AB123" si="104">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=21,MATCH($D100,$H$3:$AI$3,0)&gt;=21),1,""),"")</f>
+        <f t="shared" ref="AB100:AB123" si="104">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=21,MATCH($E100,$H$3:$AI$3,0)&gt;=21),1,""),"")</f>
         <v/>
       </c>
       <c r="AC100" s="2" t="str">
-        <f t="shared" ref="AC100:AC123" si="105">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=22,MATCH($D100,$H$3:$AI$3,0)&gt;=22),1,""),"")</f>
+        <f t="shared" ref="AC100:AC123" si="105">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=22,MATCH($E100,$H$3:$AI$3,0)&gt;=22),1,""),"")</f>
         <v/>
       </c>
       <c r="AD100" s="2" t="str">
-        <f t="shared" ref="AD100:AD123" si="106">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=23,MATCH($D100,$H$3:$AI$3,0)&gt;=23),1,""),"")</f>
+        <f t="shared" ref="AD100:AD123" si="106">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=23,MATCH($E100,$H$3:$AI$3,0)&gt;=23),1,""),"")</f>
         <v/>
       </c>
       <c r="AE100" s="2" t="str">
-        <f t="shared" ref="AE100:AE123" si="107">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=24,MATCH($D100,$H$3:$AI$3,0)&gt;=24),1,""),"")</f>
+        <f t="shared" ref="AE100:AE123" si="107">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=24,MATCH($E100,$H$3:$AI$3,0)&gt;=24),1,""),"")</f>
         <v/>
       </c>
       <c r="AF100" s="2" t="str">
-        <f t="shared" ref="AF100:AF123" si="108">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=25,MATCH($D100,$H$3:$AI$3,0)&gt;=25),1,""),"")</f>
+        <f t="shared" ref="AF100:AF123" si="108">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=25,MATCH($E100,$H$3:$AI$3,0)&gt;=25),1,""),"")</f>
         <v/>
       </c>
       <c r="AG100" s="2" t="str">
-        <f t="shared" ref="AG100:AG123" si="109">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=26,MATCH($D100,$H$3:$AI$3,0)&gt;=26),1,""),"")</f>
+        <f t="shared" ref="AG100:AG123" si="109">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=26,MATCH($E100,$H$3:$AI$3,0)&gt;=26),1,""),"")</f>
         <v/>
       </c>
       <c r="AH100" s="2" t="str">
-        <f t="shared" ref="AH100:AH123" si="110">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=27,MATCH($D100,$H$3:$AI$3,0)&gt;=27),1,""),"")</f>
+        <f t="shared" ref="AH100:AH123" si="110">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=27,MATCH($E100,$H$3:$AI$3,0)&gt;=27),1,""),"")</f>
         <v/>
       </c>
       <c r="AI100" s="14" t="str">
-        <f t="shared" ref="AI100:AI123" si="111">IFERROR(IF(AND(MATCH($C100,$H$3:$AI$3,0)&lt;=28,MATCH($D100,$H$3:$AI$3,0)&gt;=28),1,""),"")</f>
+        <f t="shared" ref="AI100:AI123" si="111">IFERROR(IF(AND(MATCH($D100,$H$3:$AI$3,0)&lt;=28,MATCH($E100,$H$3:$AI$3,0)&gt;=28),1,""),"")</f>
         <v/>
       </c>
     </row>
     <row r="101" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="19"/>
-      <c r="B101" s="20"/>
+      <c r="B101" s="16"/>
       <c r="C101" s="20"/>
       <c r="D101" s="20"/>
-      <c r="E101" s="21" t="b">
+      <c r="E101" s="20"/>
+      <c r="F101" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F101" s="19"/>
-      <c r="G101" s="16"/>
+      <c r="G101" s="19"/>
       <c r="H101" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -13243,14 +13243,14 @@
     </row>
     <row r="102" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="19"/>
-      <c r="B102" s="20"/>
+      <c r="B102" s="16"/>
       <c r="C102" s="20"/>
       <c r="D102" s="20"/>
-      <c r="E102" s="21" t="b">
+      <c r="E102" s="20"/>
+      <c r="F102" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F102" s="19"/>
-      <c r="G102" s="16"/>
+      <c r="G102" s="19"/>
       <c r="H102" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -13366,14 +13366,14 @@
     </row>
     <row r="103" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="19"/>
-      <c r="B103" s="20"/>
+      <c r="B103" s="16"/>
       <c r="C103" s="20"/>
       <c r="D103" s="20"/>
-      <c r="E103" s="21" t="b">
+      <c r="E103" s="20"/>
+      <c r="F103" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F103" s="19"/>
-      <c r="G103" s="16"/>
+      <c r="G103" s="19"/>
       <c r="H103" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -13489,14 +13489,14 @@
     </row>
     <row r="104" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="19"/>
-      <c r="B104" s="20"/>
+      <c r="B104" s="16"/>
       <c r="C104" s="20"/>
       <c r="D104" s="20"/>
-      <c r="E104" s="21" t="b">
+      <c r="E104" s="20"/>
+      <c r="F104" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F104" s="19"/>
-      <c r="G104" s="16"/>
+      <c r="G104" s="19"/>
       <c r="H104" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -13612,14 +13612,14 @@
     </row>
     <row r="105" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="19"/>
-      <c r="B105" s="20"/>
+      <c r="B105" s="16"/>
       <c r="C105" s="20"/>
       <c r="D105" s="20"/>
-      <c r="E105" s="21" t="b">
+      <c r="E105" s="20"/>
+      <c r="F105" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F105" s="19"/>
-      <c r="G105" s="16"/>
+      <c r="G105" s="19"/>
       <c r="H105" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -13735,14 +13735,14 @@
     </row>
     <row r="106" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="19"/>
-      <c r="B106" s="20"/>
+      <c r="B106" s="16"/>
       <c r="C106" s="20"/>
       <c r="D106" s="20"/>
-      <c r="E106" s="21" t="b">
+      <c r="E106" s="20"/>
+      <c r="F106" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F106" s="19"/>
-      <c r="G106" s="16"/>
+      <c r="G106" s="19"/>
       <c r="H106" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -13858,14 +13858,14 @@
     </row>
     <row r="107" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="19"/>
-      <c r="B107" s="20"/>
+      <c r="B107" s="16"/>
       <c r="C107" s="20"/>
       <c r="D107" s="20"/>
-      <c r="E107" s="21" t="b">
+      <c r="E107" s="20"/>
+      <c r="F107" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F107" s="19"/>
-      <c r="G107" s="16"/>
+      <c r="G107" s="19"/>
       <c r="H107" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -13981,14 +13981,14 @@
     </row>
     <row r="108" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="19"/>
-      <c r="B108" s="20"/>
+      <c r="B108" s="16"/>
       <c r="C108" s="20"/>
       <c r="D108" s="20"/>
-      <c r="E108" s="21" t="b">
+      <c r="E108" s="20"/>
+      <c r="F108" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F108" s="19"/>
-      <c r="G108" s="16"/>
+      <c r="G108" s="19"/>
       <c r="H108" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -14104,14 +14104,14 @@
     </row>
     <row r="109" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="19"/>
-      <c r="B109" s="20"/>
+      <c r="B109" s="16"/>
       <c r="C109" s="20"/>
       <c r="D109" s="20"/>
-      <c r="E109" s="21" t="b">
+      <c r="E109" s="20"/>
+      <c r="F109" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F109" s="19"/>
-      <c r="G109" s="16"/>
+      <c r="G109" s="19"/>
       <c r="H109" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -14227,14 +14227,14 @@
     </row>
     <row r="110" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="19"/>
-      <c r="B110" s="20"/>
+      <c r="B110" s="16"/>
       <c r="C110" s="20"/>
       <c r="D110" s="20"/>
-      <c r="E110" s="21" t="b">
+      <c r="E110" s="20"/>
+      <c r="F110" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F110" s="19"/>
-      <c r="G110" s="16"/>
+      <c r="G110" s="19"/>
       <c r="H110" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -14350,14 +14350,14 @@
     </row>
     <row r="111" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="19"/>
-      <c r="B111" s="20"/>
+      <c r="B111" s="16"/>
       <c r="C111" s="20"/>
       <c r="D111" s="20"/>
-      <c r="E111" s="21" t="b">
+      <c r="E111" s="20"/>
+      <c r="F111" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F111" s="19"/>
-      <c r="G111" s="16"/>
+      <c r="G111" s="19"/>
       <c r="H111" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -14473,14 +14473,14 @@
     </row>
     <row r="112" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="19"/>
-      <c r="B112" s="20"/>
+      <c r="B112" s="16"/>
       <c r="C112" s="20"/>
       <c r="D112" s="20"/>
-      <c r="E112" s="21" t="b">
+      <c r="E112" s="20"/>
+      <c r="F112" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F112" s="19"/>
-      <c r="G112" s="16"/>
+      <c r="G112" s="19"/>
       <c r="H112" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -14596,14 +14596,14 @@
     </row>
     <row r="113" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="19"/>
-      <c r="B113" s="20"/>
+      <c r="B113" s="16"/>
       <c r="C113" s="20"/>
       <c r="D113" s="20"/>
-      <c r="E113" s="21" t="b">
+      <c r="E113" s="20"/>
+      <c r="F113" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F113" s="19"/>
-      <c r="G113" s="16"/>
+      <c r="G113" s="19"/>
       <c r="H113" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -14719,14 +14719,14 @@
     </row>
     <row r="114" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="19"/>
-      <c r="B114" s="20"/>
+      <c r="B114" s="16"/>
       <c r="C114" s="20"/>
       <c r="D114" s="20"/>
-      <c r="E114" s="21" t="b">
+      <c r="E114" s="20"/>
+      <c r="F114" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F114" s="19"/>
-      <c r="G114" s="16"/>
+      <c r="G114" s="19"/>
       <c r="H114" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -14842,14 +14842,14 @@
     </row>
     <row r="115" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="19"/>
-      <c r="B115" s="20"/>
+      <c r="B115" s="16"/>
       <c r="C115" s="20"/>
       <c r="D115" s="20"/>
-      <c r="E115" s="21" t="b">
+      <c r="E115" s="20"/>
+      <c r="F115" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F115" s="19"/>
-      <c r="G115" s="16"/>
+      <c r="G115" s="19"/>
       <c r="H115" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -14965,14 +14965,14 @@
     </row>
     <row r="116" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="19"/>
-      <c r="B116" s="20"/>
+      <c r="B116" s="16"/>
       <c r="C116" s="20"/>
       <c r="D116" s="20"/>
-      <c r="E116" s="21" t="b">
+      <c r="E116" s="20"/>
+      <c r="F116" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F116" s="19"/>
-      <c r="G116" s="16"/>
+      <c r="G116" s="19"/>
       <c r="H116" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -15088,14 +15088,14 @@
     </row>
     <row r="117" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="19"/>
-      <c r="B117" s="20"/>
+      <c r="B117" s="16"/>
       <c r="C117" s="20"/>
       <c r="D117" s="20"/>
-      <c r="E117" s="21" t="b">
+      <c r="E117" s="20"/>
+      <c r="F117" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F117" s="19"/>
-      <c r="G117" s="16"/>
+      <c r="G117" s="19"/>
       <c r="H117" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -15211,14 +15211,14 @@
     </row>
     <row r="118" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="19"/>
-      <c r="B118" s="20"/>
+      <c r="B118" s="16"/>
       <c r="C118" s="20"/>
       <c r="D118" s="20"/>
-      <c r="E118" s="21" t="b">
+      <c r="E118" s="20"/>
+      <c r="F118" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F118" s="19"/>
-      <c r="G118" s="16"/>
+      <c r="G118" s="19"/>
       <c r="H118" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -15334,14 +15334,14 @@
     </row>
     <row r="119" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="19"/>
-      <c r="B119" s="20"/>
+      <c r="B119" s="16"/>
       <c r="C119" s="20"/>
       <c r="D119" s="20"/>
-      <c r="E119" s="21" t="b">
+      <c r="E119" s="20"/>
+      <c r="F119" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F119" s="19"/>
-      <c r="G119" s="16"/>
+      <c r="G119" s="19"/>
       <c r="H119" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -15457,14 +15457,14 @@
     </row>
     <row r="120" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="19"/>
-      <c r="B120" s="20"/>
+      <c r="B120" s="16"/>
       <c r="C120" s="20"/>
       <c r="D120" s="20"/>
-      <c r="E120" s="21" t="b">
+      <c r="E120" s="20"/>
+      <c r="F120" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F120" s="19"/>
-      <c r="G120" s="16"/>
+      <c r="G120" s="19"/>
       <c r="H120" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -15580,14 +15580,14 @@
     </row>
     <row r="121" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="19"/>
-      <c r="B121" s="20"/>
+      <c r="B121" s="16"/>
       <c r="C121" s="20"/>
       <c r="D121" s="20"/>
-      <c r="E121" s="21" t="b">
+      <c r="E121" s="20"/>
+      <c r="F121" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F121" s="19"/>
-      <c r="G121" s="16"/>
+      <c r="G121" s="19"/>
       <c r="H121" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -15703,14 +15703,14 @@
     </row>
     <row r="122" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="19"/>
-      <c r="B122" s="20"/>
+      <c r="B122" s="16"/>
       <c r="C122" s="20"/>
       <c r="D122" s="20"/>
-      <c r="E122" s="21" t="b">
+      <c r="E122" s="20"/>
+      <c r="F122" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F122" s="19"/>
-      <c r="G122" s="16"/>
+      <c r="G122" s="19"/>
       <c r="H122" s="1" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -15826,14 +15826,14 @@
     </row>
     <row r="123" spans="1:35" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="19"/>
-      <c r="B123" s="20"/>
+      <c r="B123" s="16"/>
       <c r="C123" s="20"/>
       <c r="D123" s="20"/>
-      <c r="E123" s="21" t="b">
+      <c r="E123" s="20"/>
+      <c r="F123" s="21" t="b">
         <v>0</v>
       </c>
-      <c r="F123" s="19"/>
-      <c r="G123" s="16"/>
+      <c r="G123" s="19"/>
       <c r="H123" s="3" t="str">
         <f t="shared" si="84"/>
         <v/>
@@ -15950,28 +15950,28 @@
   </sheetData>
   <sheetProtection sheet="1" selectLockedCells="1"/>
   <mergeCells count="4">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="P1:Q1"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="A4:G123">
     <cfRule type="expression" dxfId="13" priority="21">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:B123">
+  <conditionalFormatting sqref="C4:C123">
     <cfRule type="expression" dxfId="12" priority="2">
-      <formula>$B4="Not Started"</formula>
+      <formula>$C4="Not Started"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="11" priority="4">
-      <formula>$B4="In Progress"</formula>
+      <formula>$C4="In Progress"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="10" priority="7">
-      <formula>$B4="Done"</formula>
+      <formula>$C4="Done"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="9" priority="9">
-      <formula>$B4="Blocked"</formula>
+      <formula>$C4="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:AI3">
@@ -15986,19 +15986,19 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:AI123">
     <cfRule type="expression" dxfId="6" priority="10">
-      <formula>AND(H4=1,$E4=TRUE)</formula>
+      <formula>AND(H4=1,$F4=TRUE)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="5" priority="11">
-      <formula>AND(H4=1,$B4="Not Started")</formula>
+      <formula>AND(H4=1,$C4="Not Started")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="4" priority="12">
-      <formula>AND(H4=1,$B4="In Progress")</formula>
+      <formula>AND(H4=1,$C4="In Progress")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="3" priority="13">
-      <formula>AND(H4=1,$B4="Done")</formula>
+      <formula>AND(H4=1,$C4="Done")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="14">
-      <formula>AND(H4=1,$B4="Blocked")</formula>
+      <formula>AND(H4=1,$C4="Blocked")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="15">
       <formula>H4=1</formula>

</xml_diff>

<commit_message>
Fix template: unlock full title merge and realign data-validation dropdowns
- Add an unlocked B1 cell (style 27) so the whole A1:G1 title merge is
  editable — previously B1 was missing and fell back to the locked default,
  giving the merge a mixed lock state.
- Shift the three data validations by the +1 the column insert had missed:
  Status list B4:B123 -> C4:C123 (removed from Category, restored on Status),
  sprint list C4:D123 -> D4:E123 (refs $H$3:$AI$3), start-sprint list H1 -> I1.
  Category now has no dropdown.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WPLuxHLXTyjEHoQp8LTD3B
</commit_message>
<xml_diff>
--- a/assets/delivery-plan-template.xlsx
+++ b/assets/delivery-plan-template.xlsx
@@ -1016,6 +1016,7 @@
       <c r="A1" s="27" t="s">
         <v>8</v>
       </c>
+      <c r="B1" s="27"/>
       <c r="C1" s="27"/>
       <c r="D1" s="27"/>
       <c r="E1" s="27"/>
@@ -16008,16 +16009,16 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" sqref="H1" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I1" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Q1.1,Q1.2,Q1.3,Q1.4,Q1.5,Q1.6,Q1.7,Q2.1,Q2.2,Q2.3,Q2.4,Q2.5,Q2.6,Q2.7,Q3.1,Q3.2,Q3.3,Q3.4,Q3.5,Q3.6,Q3.7,Q4.1,Q4.2,Q4.3,Q4.4,Q4.5,Q4.6,Q4.7"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="B4:B123" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="C4:C123" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Not Started,In Progress,Done,Blocked"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C4:D123" xr:uid="{00000000-0002-0000-0000-000002000000}">
-      <formula1>$G$3:$AH$3</formula1>
+    <dataValidation type="list" allowBlank="1" sqref="D4:E123" xr:uid="{00000000-0002-0000-0000-000002000000}">
+      <formula1>$H$3:$AI$3</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>